<commit_message>
ROBOZÃO TÁ FICANDO SINISTRO E CHEIO DE TESTES PRONTOS PARA DEPURARMOS
</commit_message>
<xml_diff>
--- a/Comissoes_Recebimento_08_2025.xlsx
+++ b/Comissoes_Recebimento_08_2025.xlsx
@@ -2102,7 +2102,7 @@
         <v>1</v>
       </c>
       <c r="V2" s="7" t="n">
-        <v>45978.17341711806</v>
+        <v>45978.43175184027</v>
       </c>
       <c r="W2" t="inlineStr">
         <is>
@@ -2200,7 +2200,7 @@
         <v>2</v>
       </c>
       <c r="V3" s="7" t="n">
-        <v>45978.17342208333</v>
+        <v>45978.43176604166</v>
       </c>
       <c r="W3" t="inlineStr">
         <is>
@@ -2288,7 +2288,7 @@
         <v>1</v>
       </c>
       <c r="V4" s="7" t="n">
-        <v>45978.17341797454</v>
+        <v>45978.43175405093</v>
       </c>
       <c r="W4" t="inlineStr">
         <is>
@@ -2376,7 +2376,7 @@
         <v>2</v>
       </c>
       <c r="V5" s="7" t="n">
-        <v>45978.17341850694</v>
+        <v>45978.4317558449</v>
       </c>
       <c r="W5" t="inlineStr">
         <is>
@@ -2474,7 +2474,7 @@
         <v>2</v>
       </c>
       <c r="V6" s="7" t="n">
-        <v>45978.17341903935</v>
+        <v>45978.43175744213</v>
       </c>
       <c r="W6" t="inlineStr">
         <is>
@@ -2562,7 +2562,7 @@
         <v>1</v>
       </c>
       <c r="V7" s="7" t="n">
-        <v>45978.17341984954</v>
+        <v>45978.43176005787</v>
       </c>
       <c r="W7" t="inlineStr">
         <is>
@@ -2650,7 +2650,7 @@
         <v>1</v>
       </c>
       <c r="V8" s="7" t="n">
-        <v>45978.17342015047</v>
+        <v>45978.43176090278</v>
       </c>
       <c r="W8" t="inlineStr">
         <is>
@@ -2748,7 +2748,7 @@
         <v>3</v>
       </c>
       <c r="V9" s="7" t="n">
-        <v>45978.17342050926</v>
+        <v>45978.43176185185</v>
       </c>
       <c r="W9" t="inlineStr">
         <is>
@@ -2846,7 +2846,7 @@
         <v>2</v>
       </c>
       <c r="V10" s="7" t="n">
-        <v>45978.17342105324</v>
+        <v>45978.43176325232</v>
       </c>
       <c r="W10" t="inlineStr">
         <is>
@@ -2934,7 +2934,7 @@
         <v>1</v>
       </c>
       <c r="V11" s="7" t="n">
-        <v>45978.17342190972</v>
+        <v>45978.43176497685</v>
       </c>
       <c r="W11" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
ATUALIZAÇÃO 18/11 FINAL DO EXPEDIENTE
</commit_message>
<xml_diff>
--- a/Comissoes_Recebimento_08_2025.xlsx
+++ b/Comissoes_Recebimento_08_2025.xlsx
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:L28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -949,22 +949,22 @@
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>100010</t>
+          <t>100009</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>COT100010</t>
+          <t>COT100009</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>30/08/2025</t>
+          <t>18/08/2025</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>45,000.00</t>
+          <t>4,000.00</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
@@ -982,7 +982,7 @@
       <c r="I10" s="4" t="inlineStr"/>
       <c r="J10" s="4" t="inlineStr">
         <is>
-          <t>450.00</t>
+          <t>40.00</t>
         </is>
       </c>
       <c r="K10" s="4" t="inlineStr">
@@ -991,6 +991,906 @@
         </is>
       </c>
       <c r="L10" s="4" t="inlineStr">
+        <is>
+          <t>08/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>200001</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>COT200001</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>06/08/2025</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>7,500.00</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>Alessandro Cappi</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr"/>
+      <c r="G11" s="4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="H11" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I11" s="4" t="inlineStr"/>
+      <c r="J11" s="4" t="inlineStr">
+        <is>
+          <t>75.00</t>
+        </is>
+      </c>
+      <c r="K11" s="4" t="inlineStr">
+        <is>
+          <t>Adiantamento</t>
+        </is>
+      </c>
+      <c r="L11" s="4" t="inlineStr">
+        <is>
+          <t>08/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>200002</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>COT200002</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>07/08/2025</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>7,500.00</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>Alessandro Cappi</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr"/>
+      <c r="G12" s="4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="H12" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I12" s="4" t="inlineStr"/>
+      <c r="J12" s="4" t="inlineStr">
+        <is>
+          <t>75.00</t>
+        </is>
+      </c>
+      <c r="K12" s="4" t="inlineStr">
+        <is>
+          <t>Adiantamento</t>
+        </is>
+      </c>
+      <c r="L12" s="4" t="inlineStr">
+        <is>
+          <t>08/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>200003</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>COT200003</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>08/08/2025</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>7,500.00</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>Alessandro Cappi</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr"/>
+      <c r="G13" s="4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="H13" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I13" s="4" t="inlineStr"/>
+      <c r="J13" s="4" t="inlineStr">
+        <is>
+          <t>75.00</t>
+        </is>
+      </c>
+      <c r="K13" s="4" t="inlineStr">
+        <is>
+          <t>Adiantamento</t>
+        </is>
+      </c>
+      <c r="L13" s="4" t="inlineStr">
+        <is>
+          <t>08/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>200004</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>COT200004</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>09/08/2025</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>7,500.00</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>Alessandro Cappi</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr"/>
+      <c r="G14" s="4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="H14" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I14" s="4" t="inlineStr"/>
+      <c r="J14" s="4" t="inlineStr">
+        <is>
+          <t>75.00</t>
+        </is>
+      </c>
+      <c r="K14" s="4" t="inlineStr">
+        <is>
+          <t>Adiantamento</t>
+        </is>
+      </c>
+      <c r="L14" s="4" t="inlineStr">
+        <is>
+          <t>08/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>200005</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>COT200005</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>10/08/2025</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>7,500.00</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>Alessandro Cappi</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr"/>
+      <c r="G15" s="4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="H15" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I15" s="4" t="inlineStr"/>
+      <c r="J15" s="4" t="inlineStr">
+        <is>
+          <t>75.00</t>
+        </is>
+      </c>
+      <c r="K15" s="4" t="inlineStr">
+        <is>
+          <t>Adiantamento</t>
+        </is>
+      </c>
+      <c r="L15" s="4" t="inlineStr">
+        <is>
+          <t>08/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>200006</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>COT200006</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>11/08/2025</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>7,500.00</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>Alessandro Cappi</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr"/>
+      <c r="G16" s="4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="H16" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I16" s="4" t="inlineStr"/>
+      <c r="J16" s="4" t="inlineStr">
+        <is>
+          <t>75.00</t>
+        </is>
+      </c>
+      <c r="K16" s="4" t="inlineStr">
+        <is>
+          <t>Adiantamento</t>
+        </is>
+      </c>
+      <c r="L16" s="4" t="inlineStr">
+        <is>
+          <t>08/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>200015</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>COT200015</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>20/08/2025</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>6,750.00</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>Alessandro Cappi</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr"/>
+      <c r="G17" s="4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="H17" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I17" s="4" t="inlineStr"/>
+      <c r="J17" s="4" t="inlineStr">
+        <is>
+          <t>67.50</t>
+        </is>
+      </c>
+      <c r="K17" s="4" t="inlineStr">
+        <is>
+          <t>Adiantamento</t>
+        </is>
+      </c>
+      <c r="L17" s="4" t="inlineStr">
+        <is>
+          <t>08/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>200018</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>COT200018</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>23/08/2025</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>6,900.00</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>Alessandro Cappi</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr"/>
+      <c r="G18" s="4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="H18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I18" s="4" t="inlineStr"/>
+      <c r="J18" s="4" t="inlineStr">
+        <is>
+          <t>69.00</t>
+        </is>
+      </c>
+      <c r="K18" s="4" t="inlineStr">
+        <is>
+          <t>Adiantamento</t>
+        </is>
+      </c>
+      <c r="L18" s="4" t="inlineStr">
+        <is>
+          <t>08/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>200021</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>COT200021</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>06/08/2025</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>7,050.00</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>Alessandro Cappi</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr"/>
+      <c r="G19" s="4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="H19" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I19" s="4" t="inlineStr"/>
+      <c r="J19" s="4" t="inlineStr">
+        <is>
+          <t>70.50</t>
+        </is>
+      </c>
+      <c r="K19" s="4" t="inlineStr">
+        <is>
+          <t>Adiantamento</t>
+        </is>
+      </c>
+      <c r="L19" s="4" t="inlineStr">
+        <is>
+          <t>08/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>200024</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>COT200024</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>09/08/2025</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>7,200.00</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>Alessandro Cappi</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr"/>
+      <c r="G20" s="4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="H20" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I20" s="4" t="inlineStr"/>
+      <c r="J20" s="4" t="inlineStr">
+        <is>
+          <t>72.00</t>
+        </is>
+      </c>
+      <c r="K20" s="4" t="inlineStr">
+        <is>
+          <t>Adiantamento</t>
+        </is>
+      </c>
+      <c r="L20" s="4" t="inlineStr">
+        <is>
+          <t>08/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>200027</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>COT200027</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>12/08/2025</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>7,350.00</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>Alessandro Cappi</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr"/>
+      <c r="G21" s="4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="H21" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I21" s="4" t="inlineStr"/>
+      <c r="J21" s="4" t="inlineStr">
+        <is>
+          <t>73.50</t>
+        </is>
+      </c>
+      <c r="K21" s="4" t="inlineStr">
+        <is>
+          <t>Adiantamento</t>
+        </is>
+      </c>
+      <c r="L21" s="4" t="inlineStr">
+        <is>
+          <t>08/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>200030</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>COT200030</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>15/08/2025</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>7,500.00</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>Alessandro Cappi</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr"/>
+      <c r="G22" s="4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="H22" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I22" s="4" t="inlineStr"/>
+      <c r="J22" s="4" t="inlineStr">
+        <is>
+          <t>75.00</t>
+        </is>
+      </c>
+      <c r="K22" s="4" t="inlineStr">
+        <is>
+          <t>Adiantamento</t>
+        </is>
+      </c>
+      <c r="L22" s="4" t="inlineStr">
+        <is>
+          <t>08/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>200033</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>COT200033</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>18/08/2025</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>7,650.00</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>Alessandro Cappi</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr"/>
+      <c r="G23" s="4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="H23" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I23" s="4" t="inlineStr"/>
+      <c r="J23" s="4" t="inlineStr">
+        <is>
+          <t>76.50</t>
+        </is>
+      </c>
+      <c r="K23" s="4" t="inlineStr">
+        <is>
+          <t>Adiantamento</t>
+        </is>
+      </c>
+      <c r="L23" s="4" t="inlineStr">
+        <is>
+          <t>08/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>200036</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>COT200036</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>21/08/2025</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>7,800.00</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>Alessandro Cappi</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr"/>
+      <c r="G24" s="4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="H24" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I24" s="4" t="inlineStr"/>
+      <c r="J24" s="4" t="inlineStr">
+        <is>
+          <t>78.00</t>
+        </is>
+      </c>
+      <c r="K24" s="4" t="inlineStr">
+        <is>
+          <t>Adiantamento</t>
+        </is>
+      </c>
+      <c r="L24" s="4" t="inlineStr">
+        <is>
+          <t>08/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>200039</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>COT200039</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>24/08/2025</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>7,950.00</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>Alessandro Cappi</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr"/>
+      <c r="G25" s="4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="H25" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I25" s="4" t="inlineStr"/>
+      <c r="J25" s="4" t="inlineStr">
+        <is>
+          <t>79.50</t>
+        </is>
+      </c>
+      <c r="K25" s="4" t="inlineStr">
+        <is>
+          <t>Adiantamento</t>
+        </is>
+      </c>
+      <c r="L25" s="4" t="inlineStr">
+        <is>
+          <t>08/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>200042</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>COT200042</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>07/08/2025</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>8,100.00</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>Alessandro Cappi</t>
+        </is>
+      </c>
+      <c r="F26" s="4" t="inlineStr"/>
+      <c r="G26" s="4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="H26" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I26" s="4" t="inlineStr"/>
+      <c r="J26" s="4" t="inlineStr">
+        <is>
+          <t>81.00</t>
+        </is>
+      </c>
+      <c r="K26" s="4" t="inlineStr">
+        <is>
+          <t>Adiantamento</t>
+        </is>
+      </c>
+      <c r="L26" s="4" t="inlineStr">
+        <is>
+          <t>08/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>200045</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>COT200045</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>10/08/2025</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>8,250.00</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>Alessandro Cappi</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="inlineStr"/>
+      <c r="G27" s="4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="H27" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I27" s="4" t="inlineStr"/>
+      <c r="J27" s="4" t="inlineStr">
+        <is>
+          <t>82.50</t>
+        </is>
+      </c>
+      <c r="K27" s="4" t="inlineStr">
+        <is>
+          <t>Adiantamento</t>
+        </is>
+      </c>
+      <c r="L27" s="4" t="inlineStr">
+        <is>
+          <t>08/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>200048</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>COT200048</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>13/08/2025</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>8,400.00</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="inlineStr">
+        <is>
+          <t>Alessandro Cappi</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="inlineStr"/>
+      <c r="G28" s="4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="H28" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I28" s="4" t="inlineStr"/>
+      <c r="J28" s="4" t="inlineStr">
+        <is>
+          <t>84.00</t>
+        </is>
+      </c>
+      <c r="K28" s="4" t="inlineStr">
+        <is>
+          <t>Adiantamento</t>
+        </is>
+      </c>
+      <c r="L28" s="4" t="inlineStr">
         <is>
           <t>08/2025</t>
         </is>
@@ -1007,7 +1907,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M13"/>
+  <dimension ref="A1:M9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1124,11 +2024,11 @@
       </c>
       <c r="H2" s="5" t="inlineStr"/>
       <c r="I2" s="5" t="n">
-        <v>0.4531463210515605</v>
+        <v>0.2400860712068003</v>
       </c>
       <c r="J2" s="5" t="inlineStr">
         <is>
-          <t>33.99</t>
+          <t>18.01</t>
         </is>
       </c>
       <c r="K2" s="5" t="inlineStr">
@@ -1179,11 +2079,11 @@
       </c>
       <c r="H3" s="5" t="inlineStr"/>
       <c r="I3" s="5" t="n">
-        <v>0.4813732900296912</v>
+        <v>0.2821262377699738</v>
       </c>
       <c r="J3" s="5" t="inlineStr">
         <is>
-          <t>28.88</t>
+          <t>16.93</t>
         </is>
       </c>
       <c r="K3" s="5" t="inlineStr">
@@ -1234,11 +2134,11 @@
       </c>
       <c r="H4" s="5" t="inlineStr"/>
       <c r="I4" s="5" t="n">
-        <v>0.4813732900296912</v>
+        <v>0.2821262377699738</v>
       </c>
       <c r="J4" s="5" t="inlineStr">
         <is>
-          <t>28.88</t>
+          <t>16.93</t>
         </is>
       </c>
       <c r="K4" s="5" t="inlineStr">
@@ -1289,11 +2189,11 @@
       </c>
       <c r="H5" s="5" t="inlineStr"/>
       <c r="I5" s="5" t="n">
-        <v>0.3313732900296912</v>
+        <v>0.2821262377699738</v>
       </c>
       <c r="J5" s="5" t="inlineStr">
         <is>
-          <t>19.88</t>
+          <t>16.93</t>
         </is>
       </c>
       <c r="K5" s="5" t="inlineStr">
@@ -1344,11 +2244,11 @@
       </c>
       <c r="H6" s="5" t="inlineStr"/>
       <c r="I6" s="5" t="n">
-        <v>0.3313732900296912</v>
+        <v>0.2821262377699738</v>
       </c>
       <c r="J6" s="5" t="inlineStr">
         <is>
-          <t>19.88</t>
+          <t>16.93</t>
         </is>
       </c>
       <c r="K6" s="5" t="inlineStr">
@@ -1399,11 +2299,11 @@
       </c>
       <c r="H7" s="5" t="inlineStr"/>
       <c r="I7" s="5" t="n">
-        <v>0.4531463210515605</v>
+        <v>0.2400860712068003</v>
       </c>
       <c r="J7" s="5" t="inlineStr">
         <is>
-          <t>67.97</t>
+          <t>36.01</t>
         </is>
       </c>
       <c r="K7" s="5" t="inlineStr">
@@ -1454,11 +2354,11 @@
       </c>
       <c r="H8" s="5" t="inlineStr"/>
       <c r="I8" s="5" t="n">
-        <v>0.4531463210515605</v>
+        <v>0.2400860712068003</v>
       </c>
       <c r="J8" s="5" t="inlineStr">
         <is>
-          <t>90.63</t>
+          <t>48.02</t>
         </is>
       </c>
       <c r="K8" s="5" t="inlineStr">
@@ -1509,11 +2409,11 @@
       </c>
       <c r="H9" s="5" t="inlineStr"/>
       <c r="I9" s="5" t="n">
-        <v>0.4531463210515605</v>
+        <v>0.2400860712068003</v>
       </c>
       <c r="J9" s="5" t="inlineStr">
         <is>
-          <t>67.97</t>
+          <t>36.01</t>
         </is>
       </c>
       <c r="K9" s="5" t="inlineStr">
@@ -1527,226 +2427,6 @@
         </is>
       </c>
       <c r="M9" s="5" t="inlineStr">
-        <is>
-          <t>08/2025</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>100009</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>12345</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>20/08/2025</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>4,000.00</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t>Alessandro Cappi</t>
-        </is>
-      </c>
-      <c r="F10" s="5" t="inlineStr"/>
-      <c r="G10" s="5" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="H10" s="5" t="inlineStr"/>
-      <c r="I10" s="5" t="n">
-        <v>0.4699623876768299</v>
-      </c>
-      <c r="J10" s="5" t="inlineStr">
-        <is>
-          <t>18.80</t>
-        </is>
-      </c>
-      <c r="K10" s="5" t="inlineStr">
-        <is>
-          <t>Pagamento Regular</t>
-        </is>
-      </c>
-      <c r="L10" s="5" t="inlineStr">
-        <is>
-          <t>08/2025</t>
-        </is>
-      </c>
-      <c r="M10" s="5" t="inlineStr">
-        <is>
-          <t>08/2025</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>100009</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>12345</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>25/08/2025</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>4,000.00</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t>Alessandro Cappi</t>
-        </is>
-      </c>
-      <c r="F11" s="5" t="inlineStr"/>
-      <c r="G11" s="5" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="H11" s="5" t="inlineStr"/>
-      <c r="I11" s="5" t="n">
-        <v>0.4699623876768299</v>
-      </c>
-      <c r="J11" s="5" t="inlineStr">
-        <is>
-          <t>18.80</t>
-        </is>
-      </c>
-      <c r="K11" s="5" t="inlineStr">
-        <is>
-          <t>Pagamento Regular</t>
-        </is>
-      </c>
-      <c r="L11" s="5" t="inlineStr">
-        <is>
-          <t>08/2025</t>
-        </is>
-      </c>
-      <c r="M11" s="5" t="inlineStr">
-        <is>
-          <t>08/2025</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>100009</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>12345</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>20/08/2025</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>4,000.00</t>
-        </is>
-      </c>
-      <c r="E12" s="5" t="inlineStr">
-        <is>
-          <t>André Caramello</t>
-        </is>
-      </c>
-      <c r="F12" s="5" t="inlineStr"/>
-      <c r="G12" s="5" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="H12" s="5" t="inlineStr"/>
-      <c r="I12" s="5" t="n">
-        <v>0.3199623876768299</v>
-      </c>
-      <c r="J12" s="5" t="inlineStr">
-        <is>
-          <t>12.80</t>
-        </is>
-      </c>
-      <c r="K12" s="5" t="inlineStr">
-        <is>
-          <t>Pagamento Regular</t>
-        </is>
-      </c>
-      <c r="L12" s="5" t="inlineStr">
-        <is>
-          <t>08/2025</t>
-        </is>
-      </c>
-      <c r="M12" s="5" t="inlineStr">
-        <is>
-          <t>08/2025</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="5" t="inlineStr">
-        <is>
-          <t>100009</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>12345</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>25/08/2025</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>4,000.00</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>André Caramello</t>
-        </is>
-      </c>
-      <c r="F13" s="5" t="inlineStr"/>
-      <c r="G13" s="5" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="H13" s="5" t="inlineStr"/>
-      <c r="I13" s="5" t="n">
-        <v>0.3199623876768299</v>
-      </c>
-      <c r="J13" s="5" t="inlineStr">
-        <is>
-          <t>12.80</t>
-        </is>
-      </c>
-      <c r="K13" s="5" t="inlineStr">
-        <is>
-          <t>Pagamento Regular</t>
-        </is>
-      </c>
-      <c r="L13" s="5" t="inlineStr">
-        <is>
-          <t>08/2025</t>
-        </is>
-      </c>
-      <c r="M13" s="5" t="inlineStr">
         <is>
           <t>08/2025</t>
         </is>
@@ -1839,19 +2519,19 @@
         <v>0.01</v>
       </c>
       <c r="D2" s="6" t="n">
-        <v>0.453146</v>
+        <v>0.240086</v>
       </c>
       <c r="E2" s="6" t="n">
         <v>75</v>
       </c>
       <c r="F2" s="6" t="n">
-        <v>33.985974</v>
+        <v>18.006455</v>
       </c>
       <c r="G2" s="6" t="n">
-        <v>-0.546854</v>
+        <v>-0.759914</v>
       </c>
       <c r="H2" s="6" t="n">
-        <v>-41.014026</v>
+        <v>-56.993545</v>
       </c>
       <c r="I2" s="6" t="inlineStr">
         <is>
@@ -1870,7 +2550,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y11"/>
+  <dimension ref="A1:Y28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2102,7 +2782,7 @@
         <v>1</v>
       </c>
       <c r="V2" s="7" t="n">
-        <v>45978.43175184027</v>
+        <v>45979.55424372685</v>
       </c>
       <c r="W2" t="inlineStr">
         <is>
@@ -2140,10 +2820,10 @@
         <v>75.00000000000001</v>
       </c>
       <c r="H3" t="n">
-        <v>33.98597407886705</v>
+        <v>18.00645534051003</v>
       </c>
       <c r="I3" t="n">
-        <v>108.9859740788671</v>
+        <v>93.00645534051004</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
@@ -2172,17 +2852,17 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>{"Alessandro Cappi": 0.4531463210515605}</t>
+          <t>{"Alessandro Cappi": 0.24008607120680028}</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>{"Alessandro Cappi": {"itens": [{"negocio": "SSO", "grupo": "Analisador Fixo", "subgrupo": "Falco", "tipo_mercadoria": "Produto", "valor": 15000.0, "taxa": 0.010000000000000002, "fc": 0.4531463210515605, "taxa_rateio": 0.05, "fatia_cargo": 0.2, "fc_detalhes": {"componentes": [{"nome_meta": "Faturamento da Linha", "peso": 0.15, "realizado": 85000.0, "meta": 100.0, "atingimento": 850.0, "atingimento_cap": 1.0, "componente_fc": 0.15}, {"nome_meta": "Conversão da Linha", "peso": 0.3, "realizado": 0.0, "meta": 100.0, "atingimento": 0.0, "atingimento_cap": 0.0, "componente_fc": 0.0}, {"nome_meta": "Rentabilidade", "peso": 0.2, "realizado": 0.255, "meta": 0.3330148556610093, "atingimento": 0.7657316052578024, "atingimento_cap": 0.7657316052578024, "componente_fc": 0.15314632105156048}, {"nome_meta": "Retenção de Clientes", "peso": 0.15, "realizado": 1.0, "meta": 0.0, "atingimento": 1.0, "atingimento_cap": 1.0, "componente_fc": 0.15}, {"nome_meta": "Meta Fornecedor 2", "peso": 0.1, "realizado": 0.0, "meta": 66.66666666666667, "atingimento": 0.0, "atingimento_cap": 0.0, "componente_fc": 0.0}], "fc_total": 0.4531463210515605}}], "total_valor": 15000.0, "soma_ponderada": 150.00000000000003, "tcmp_final": 0.010000000000000002}}</t>
+          <t>{"Alessandro Cappi": {"itens": [{"negocio": "SSO", "grupo": "Analisador Fixo", "subgrupo": "Falco", "tipo_mercadoria": "Produto", "valor": 15000.0, "taxa": 0.010000000000000002, "fc": 0.24008607120680028, "taxa_rateio": 0.05, "fatia_cargo": 0.2, "fc_detalhes": {"componentes": [{"nome_meta": "Faturamento da Linha", "peso": 0.15, "realizado": 412500.0, "meta": 0.0, "atingimento": 1.0, "atingimento_cap": 1.0, "componente_fc": 0.15}, {"nome_meta": "Conversão da Linha", "peso": 0.3, "realizado": 0.0, "meta": 0.0, "atingimento": 0.0, "atingimento_cap": 0.0, "componente_fc": 0.0}, {"nome_meta": "Rentabilidade", "peso": 0.2, "realizado": 0.15, "meta": 0.3330148556610093, "atingimento": 0.4504303560340014, "atingimento_cap": 0.4504303560340014, "componente_fc": 0.09008607120680029}, {"nome_meta": "Meta Fornecedor 2", "peso": 0.1, "realizado": 4370.56, "meta": 66.66666666666667, "atingimento": 65.5584, "atingimento_cap": 1.0, "componente_fc": 0.1}], "fc_total": 0.24008607120680028}}], "total_valor": 15000.0, "soma_ponderada": 150.00000000000003, "tcmp_final": 0.010000000000000002}}</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>{"Alessandro Cappi": {"itens": [{"negocio": "SSO", "grupo": "Analisador Fixo", "subgrupo": "Falco", "tipo_mercadoria": "Produto", "valor": 15000.0, "taxa": 0.010000000000000002, "fc": 0.4531463210515605, "taxa_rateio": 0.05, "fatia_cargo": 0.2, "fc_detalhes": {"componentes": [{"nome_meta": "Faturamento da Linha", "peso": 0.15, "realizado": 85000.0, "meta": 100.0, "atingimento": 850.0, "atingimento_cap": 1.0, "componente_fc": 0.15}, {"nome_meta": "Conversão da Linha", "peso": 0.3, "realizado": 0.0, "meta": 100.0, "atingimento": 0.0, "atingimento_cap": 0.0, "componente_fc": 0.0}, {"nome_meta": "Rentabilidade", "peso": 0.2, "realizado": 0.255, "meta": 0.3330148556610093, "atingimento": 0.7657316052578024, "atingimento_cap": 0.7657316052578024, "componente_fc": 0.15314632105156048}, {"nome_meta": "Retenção de Clientes", "peso": 0.15, "realizado": 1.0, "meta": 0.0, "atingimento": 1.0, "atingimento_cap": 1.0, "componente_fc": 0.15}, {"nome_meta": "Meta Fornecedor 2", "peso": 0.1, "realizado": 0.0, "meta": 66.66666666666667, "atingimento": 0.0, "atingimento_cap": 0.0, "componente_fc": 0.0}], "fc_total": 0.4531463210515605}}], "total_valor": 15000.0, "soma_ponderada": 6797.194815773408, "fcmp_final": 0.4531463210515605}}</t>
+          <t>{"Alessandro Cappi": {"itens": [{"negocio": "SSO", "grupo": "Analisador Fixo", "subgrupo": "Falco", "tipo_mercadoria": "Produto", "valor": 15000.0, "taxa": 0.010000000000000002, "fc": 0.24008607120680028, "taxa_rateio": 0.05, "fatia_cargo": 0.2, "fc_detalhes": {"componentes": [{"nome_meta": "Faturamento da Linha", "peso": 0.15, "realizado": 412500.0, "meta": 0.0, "atingimento": 1.0, "atingimento_cap": 1.0, "componente_fc": 0.15}, {"nome_meta": "Conversão da Linha", "peso": 0.3, "realizado": 0.0, "meta": 0.0, "atingimento": 0.0, "atingimento_cap": 0.0, "componente_fc": 0.0}, {"nome_meta": "Rentabilidade", "peso": 0.2, "realizado": 0.15, "meta": 0.3330148556610093, "atingimento": 0.4504303560340014, "atingimento_cap": 0.4504303560340014, "componente_fc": 0.09008607120680029}, {"nome_meta": "Meta Fornecedor 2", "peso": 0.1, "realizado": 4370.56, "meta": 66.66666666666667, "atingimento": 65.5584, "atingimento_cap": 1.0, "componente_fc": 0.1}], "fc_total": 0.24008607120680028}}], "total_valor": 15000.0, "soma_ponderada": 3601.2910681020044, "fcmp_final": 0.24008607120680028}}</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
@@ -2200,7 +2880,7 @@
         <v>2</v>
       </c>
       <c r="V3" s="7" t="n">
-        <v>45978.43176604166</v>
+        <v>45979.55425841435</v>
       </c>
       <c r="W3" t="inlineStr">
         <is>
@@ -2288,7 +2968,7 @@
         <v>1</v>
       </c>
       <c r="V4" s="7" t="n">
-        <v>45978.43175405093</v>
+        <v>45979.55424490741</v>
       </c>
       <c r="W4" t="inlineStr">
         <is>
@@ -2376,7 +3056,7 @@
         <v>2</v>
       </c>
       <c r="V5" s="7" t="n">
-        <v>45978.4317558449</v>
+        <v>45979.55424552083</v>
       </c>
       <c r="W5" t="inlineStr">
         <is>
@@ -2414,10 +3094,10 @@
         <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>97.52958960712591</v>
+        <v>67.71029706479372</v>
       </c>
       <c r="I6" t="n">
-        <v>97.52958960712591</v>
+        <v>67.71029706479372</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
@@ -2446,17 +3126,17 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>{"André Caramello": 0.33137329002969124, "Alessandro Cappi": 0.4813732900296912}</t>
+          <t>{"André Caramello": 0.28212623776997375, "Alessandro Cappi": 0.28212623776997375}</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>{"André Caramello": {"itens": [{"negocio": "SSO", "grupo": "Analisador Portátil", "subgrupo": "Acessório", "tipo_mercadoria": "Produto", "valor": 12000.0, "taxa": 0.010000000000000002, "fc": 0.33137329002969124, "taxa_rateio": 0.05, "fatia_cargo": 0.2, "fc_detalhes": {"componentes": [{"nome_meta": "Faturamento da Linha", "peso": 0.15, "realizado": 85000.0, "meta": 100.0, "atingimento": 850.0, "atingimento_cap": 1.0, "componente_fc": 0.15}, {"nome_meta": "Conversão da Linha", "peso": 0.3, "realizado": 0.0, "meta": 100.0, "atingimento": 0.0, "atingimento_cap": 0.0, "componente_fc": 0.0}, {"nome_meta": "Rentabilidade", "peso": 0.2, "realizado": 0.302, "meta": 0.3330148556610093, "atingimento": 0.9068664501484561, "atingimento_cap": 0.9068664501484561, "componente_fc": 0.18137329002969124}, {"nome_meta": "Meta Fornecedor 2", "peso": 0.1, "realizado": 0.0, "meta": 66.66666666666667, "atingimento": 0.0, "atingimento_cap": 0.0, "componente_fc": 0.0}], "fc_total": 0.33137329002969124}}], "total_valor": 12000.0, "soma_ponderada": 120.00000000000003, "tcmp_final": 0.010000000000000002}, "Alessandro Cappi": {"itens": [{"negocio": "SSO", "grupo": "Analisador Portátil", "subgrupo": "Acessório", "tipo_mercadoria": "Produto", "valor": 12000.0, "taxa": 0.010000000000000002, "fc": 0.4813732900296912, "taxa_rateio": 0.05, "fatia_cargo": 0.2, "fc_detalhes": {"componentes": [{"nome_meta": "Faturamento da Linha", "peso": 0.15, "realizado": 85000.0, "meta": 100.0, "atingimento": 850.0, "atingimento_cap": 1.0, "componente_fc": 0.15}, {"nome_meta": "Conversão da Linha", "peso": 0.3, "realizado": 0.0, "meta": 100.0, "atingimento": 0.0, "atingimento_cap": 0.0, "componente_fc": 0.0}, {"nome_meta": "Rentabilidade", "peso": 0.2, "realizado": 0.302, "meta": 0.3330148556610093, "atingimento": 0.9068664501484561, "atingimento_cap": 0.9068664501484561, "componente_fc": 0.18137329002969124}, {"nome_meta": "Retenção de Clientes", "peso": 0.15, "realizado": 1.0, "meta": 0.0, "atingimento": 1.0, "atingimento_cap": 1.0, "componente_fc": 0.15}, {"nome_meta": "Meta Fornecedor 2", "peso": 0.1, "realizado": 0.0, "meta": 66.66666666666667, "atingimento": 0.0, "atingimento_cap": 0.0, "componente_fc": 0.0}], "fc_total": 0.4813732900296912}}], "total_valor": 12000.0, "soma_ponderada": 120.00000000000003, "tcmp_final": 0.010000000000000002}}</t>
+          <t>{"André Caramello": {"itens": [{"negocio": "SSO", "grupo": "Analisador Portátil", "subgrupo": "Acessório", "tipo_mercadoria": "Produto", "valor": 12000.0, "taxa": 0.010000000000000002, "fc": 0.28212623776997375, "taxa_rateio": 0.05, "fatia_cargo": 0.2, "fc_detalhes": {"componentes": [{"nome_meta": "Faturamento da Linha", "peso": 0.15, "realizado": 412500.0, "meta": 0.0, "atingimento": 1.0, "atingimento_cap": 1.0, "componente_fc": 0.15}, {"nome_meta": "Conversão da Linha", "peso": 0.3, "realizado": 0.0, "meta": 0.0, "atingimento": 0.0, "atingimento_cap": 0.0, "componente_fc": 0.0}, {"nome_meta": "Rentabilidade", "peso": 0.2, "realizado": 0.22, "meta": 0.3330148556610093, "atingimento": 0.6606311888498687, "atingimento_cap": 0.6606311888498687, "componente_fc": 0.13212623776997376}, {"nome_meta": "Meta Fornecedor 2", "peso": 0.1, "realizado": 4370.56, "meta": 66.66666666666667, "atingimento": 65.5584, "atingimento_cap": 1.0, "componente_fc": 0.1}], "fc_total": 0.28212623776997375}}], "total_valor": 12000.0, "soma_ponderada": 120.00000000000003, "tcmp_final": 0.010000000000000002}, "Alessandro Cappi": {"itens": [{"negocio": "SSO", "grupo": "Analisador Portátil", "subgrupo": "Acessório", "tipo_mercadoria": "Produto", "valor": 12000.0, "taxa": 0.010000000000000002, "fc": 0.28212623776997375, "taxa_rateio": 0.05, "fatia_cargo": 0.2, "fc_detalhes": {"componentes": [{"nome_meta": "Faturamento da Linha", "peso": 0.15, "realizado": 412500.0, "meta": 0.0, "atingimento": 1.0, "atingimento_cap": 1.0, "componente_fc": 0.15}, {"nome_meta": "Conversão da Linha", "peso": 0.3, "realizado": 0.0, "meta": 0.0, "atingimento": 0.0, "atingimento_cap": 0.0, "componente_fc": 0.0}, {"nome_meta": "Rentabilidade", "peso": 0.2, "realizado": 0.22, "meta": 0.3330148556610093, "atingimento": 0.6606311888498687, "atingimento_cap": 0.6606311888498687, "componente_fc": 0.13212623776997376}, {"nome_meta": "Meta Fornecedor 2", "peso": 0.1, "realizado": 4370.56, "meta": 66.66666666666667, "atingimento": 65.5584, "atingimento_cap": 1.0, "componente_fc": 0.1}], "fc_total": 0.28212623776997375}}], "total_valor": 12000.0, "soma_ponderada": 120.00000000000003, "tcmp_final": 0.010000000000000002}}</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>{"André Caramello": {"itens": [{"negocio": "SSO", "grupo": "Analisador Portátil", "subgrupo": "Acessório", "tipo_mercadoria": "Produto", "valor": 12000.0, "taxa": 0.010000000000000002, "fc": 0.33137329002969124, "taxa_rateio": 0.05, "fatia_cargo": 0.2, "fc_detalhes": {"componentes": [{"nome_meta": "Faturamento da Linha", "peso": 0.15, "realizado": 85000.0, "meta": 100.0, "atingimento": 850.0, "atingimento_cap": 1.0, "componente_fc": 0.15}, {"nome_meta": "Conversão da Linha", "peso": 0.3, "realizado": 0.0, "meta": 100.0, "atingimento": 0.0, "atingimento_cap": 0.0, "componente_fc": 0.0}, {"nome_meta": "Rentabilidade", "peso": 0.2, "realizado": 0.302, "meta": 0.3330148556610093, "atingimento": 0.9068664501484561, "atingimento_cap": 0.9068664501484561, "componente_fc": 0.18137329002969124}, {"nome_meta": "Meta Fornecedor 2", "peso": 0.1, "realizado": 0.0, "meta": 66.66666666666667, "atingimento": 0.0, "atingimento_cap": 0.0, "componente_fc": 0.0}], "fc_total": 0.33137329002969124}}], "total_valor": 12000.0, "soma_ponderada": 3976.479480356295, "fcmp_final": 0.33137329002969124}, "Alessandro Cappi": {"itens": [{"negocio": "SSO", "grupo": "Analisador Portátil", "subgrupo": "Acessório", "tipo_mercadoria": "Produto", "valor": 12000.0, "taxa": 0.010000000000000002, "fc": 0.4813732900296912, "taxa_rateio": 0.05, "fatia_cargo": 0.2, "fc_detalhes": {"componentes": [{"nome_meta": "Faturamento da Linha", "peso": 0.15, "realizado": 85000.0, "meta": 100.0, "atingimento": 850.0, "atingimento_cap": 1.0, "componente_fc": 0.15}, {"nome_meta": "Conversão da Linha", "peso": 0.3, "realizado": 0.0, "meta": 100.0, "atingimento": 0.0, "atingimento_cap": 0.0, "componente_fc": 0.0}, {"nome_meta": "Rentabilidade", "peso": 0.2, "realizado": 0.302, "meta": 0.3330148556610093, "atingimento": 0.9068664501484561, "atingimento_cap": 0.9068664501484561, "componente_fc": 0.18137329002969124}, {"nome_meta": "Retenção de Clientes", "peso": 0.15, "realizado": 1.0, "meta": 0.0, "atingimento": 1.0, "atingimento_cap": 1.0, "componente_fc": 0.15}, {"nome_meta": "Meta Fornecedor 2", "peso": 0.1, "realizado": 0.0, "meta": 66.66666666666667, "atingimento": 0.0, "atingimento_cap": 0.0, "componente_fc": 0.0}], "fc_total": 0.4813732900296912}}], "total_valor": 12000.0, "soma_ponderada": 5776.4794803562945, "fcmp_final": 0.4813732900296912}}</t>
+          <t>{"André Caramello": {"itens": [{"negocio": "SSO", "grupo": "Analisador Portátil", "subgrupo": "Acessório", "tipo_mercadoria": "Produto", "valor": 12000.0, "taxa": 0.010000000000000002, "fc": 0.28212623776997375, "taxa_rateio": 0.05, "fatia_cargo": 0.2, "fc_detalhes": {"componentes": [{"nome_meta": "Faturamento da Linha", "peso": 0.15, "realizado": 412500.0, "meta": 0.0, "atingimento": 1.0, "atingimento_cap": 1.0, "componente_fc": 0.15}, {"nome_meta": "Conversão da Linha", "peso": 0.3, "realizado": 0.0, "meta": 0.0, "atingimento": 0.0, "atingimento_cap": 0.0, "componente_fc": 0.0}, {"nome_meta": "Rentabilidade", "peso": 0.2, "realizado": 0.22, "meta": 0.3330148556610093, "atingimento": 0.6606311888498687, "atingimento_cap": 0.6606311888498687, "componente_fc": 0.13212623776997376}, {"nome_meta": "Meta Fornecedor 2", "peso": 0.1, "realizado": 4370.56, "meta": 66.66666666666667, "atingimento": 65.5584, "atingimento_cap": 1.0, "componente_fc": 0.1}], "fc_total": 0.28212623776997375}}], "total_valor": 12000.0, "soma_ponderada": 3385.514853239685, "fcmp_final": 0.28212623776997375}, "Alessandro Cappi": {"itens": [{"negocio": "SSO", "grupo": "Analisador Portátil", "subgrupo": "Acessório", "tipo_mercadoria": "Produto", "valor": 12000.0, "taxa": 0.010000000000000002, "fc": 0.28212623776997375, "taxa_rateio": 0.05, "fatia_cargo": 0.2, "fc_detalhes": {"componentes": [{"nome_meta": "Faturamento da Linha", "peso": 0.15, "realizado": 412500.0, "meta": 0.0, "atingimento": 1.0, "atingimento_cap": 1.0, "componente_fc": 0.15}, {"nome_meta": "Conversão da Linha", "peso": 0.3, "realizado": 0.0, "meta": 0.0, "atingimento": 0.0, "atingimento_cap": 0.0, "componente_fc": 0.0}, {"nome_meta": "Rentabilidade", "peso": 0.2, "realizado": 0.22, "meta": 0.3330148556610093, "atingimento": 0.6606311888498687, "atingimento_cap": 0.6606311888498687, "componente_fc": 0.13212623776997376}, {"nome_meta": "Meta Fornecedor 2", "peso": 0.1, "realizado": 4370.56, "meta": 66.66666666666667, "atingimento": 65.5584, "atingimento_cap": 1.0, "componente_fc": 0.1}], "fc_total": 0.28212623776997375}}], "total_valor": 12000.0, "soma_ponderada": 3385.514853239685, "fcmp_final": 0.28212623776997375}}</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
@@ -2474,7 +3154,7 @@
         <v>2</v>
       </c>
       <c r="V6" s="7" t="n">
-        <v>45978.43175744213</v>
+        <v>45979.5542462963</v>
       </c>
       <c r="W6" t="inlineStr">
         <is>
@@ -2562,7 +3242,7 @@
         <v>1</v>
       </c>
       <c r="V7" s="7" t="n">
-        <v>45978.43176005787</v>
+        <v>45979.55424871528</v>
       </c>
       <c r="W7" t="inlineStr">
         <is>
@@ -2650,7 +3330,7 @@
         <v>1</v>
       </c>
       <c r="V8" s="7" t="n">
-        <v>45978.43176090278</v>
+        <v>45979.55424935185</v>
       </c>
       <c r="W8" t="inlineStr">
         <is>
@@ -2688,10 +3368,10 @@
         <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>226.5731605257803</v>
+        <v>120.0430356034002</v>
       </c>
       <c r="I9" t="n">
-        <v>226.5731605257803</v>
+        <v>120.0430356034002</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
@@ -2720,17 +3400,17 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>{"Alessandro Cappi": 0.4531463210515605}</t>
+          <t>{"Alessandro Cappi": 0.2400860712068003}</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>{"Alessandro Cappi": {"itens": [{"negocio": "SSO", "grupo": "Analisador Fixo", "subgrupo": "Falco", "tipo_mercadoria": "Produto", "valor": 50000.0, "taxa": 0.010000000000000002, "fc": 0.4531463210515605, "taxa_rateio": 0.05, "fatia_cargo": 0.2, "fc_detalhes": {"componentes": [{"nome_meta": "Faturamento da Linha", "peso": 0.15, "realizado": 85000.0, "meta": 100.0, "atingimento": 850.0, "atingimento_cap": 1.0, "componente_fc": 0.15}, {"nome_meta": "Conversão da Linha", "peso": 0.3, "realizado": 0.0, "meta": 100.0, "atingimento": 0.0, "atingimento_cap": 0.0, "componente_fc": 0.0}, {"nome_meta": "Rentabilidade", "peso": 0.2, "realizado": 0.255, "meta": 0.3330148556610093, "atingimento": 0.7657316052578024, "atingimento_cap": 0.7657316052578024, "componente_fc": 0.15314632105156048}, {"nome_meta": "Retenção de Clientes", "peso": 0.15, "realizado": 1.0, "meta": 0.0, "atingimento": 1.0, "atingimento_cap": 1.0, "componente_fc": 0.15}, {"nome_meta": "Meta Fornecedor 2", "peso": 0.1, "realizado": 0.0, "meta": 66.66666666666667, "atingimento": 0.0, "atingimento_cap": 0.0, "componente_fc": 0.0}], "fc_total": 0.4531463210515605}}], "total_valor": 50000.0, "soma_ponderada": 500.0000000000001, "tcmp_final": 0.010000000000000002}}</t>
+          <t>{"Alessandro Cappi": {"itens": [{"negocio": "SSO", "grupo": "Analisador Fixo", "subgrupo": "Falco", "tipo_mercadoria": "Produto", "valor": 50000.0, "taxa": 0.010000000000000002, "fc": 0.24008607120680028, "taxa_rateio": 0.05, "fatia_cargo": 0.2, "fc_detalhes": {"componentes": [{"nome_meta": "Faturamento da Linha", "peso": 0.15, "realizado": 412500.0, "meta": 0.0, "atingimento": 1.0, "atingimento_cap": 1.0, "componente_fc": 0.15}, {"nome_meta": "Conversão da Linha", "peso": 0.3, "realizado": 0.0, "meta": 0.0, "atingimento": 0.0, "atingimento_cap": 0.0, "componente_fc": 0.0}, {"nome_meta": "Rentabilidade", "peso": 0.2, "realizado": 0.15, "meta": 0.3330148556610093, "atingimento": 0.4504303560340014, "atingimento_cap": 0.4504303560340014, "componente_fc": 0.09008607120680029}, {"nome_meta": "Meta Fornecedor 2", "peso": 0.1, "realizado": 4370.56, "meta": 66.66666666666667, "atingimento": 65.5584, "atingimento_cap": 1.0, "componente_fc": 0.1}], "fc_total": 0.24008607120680028}}], "total_valor": 50000.0, "soma_ponderada": 500.0000000000001, "tcmp_final": 0.010000000000000002}}</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>{"Alessandro Cappi": {"itens": [{"negocio": "SSO", "grupo": "Analisador Fixo", "subgrupo": "Falco", "tipo_mercadoria": "Produto", "valor": 50000.0, "taxa": 0.010000000000000002, "fc": 0.4531463210515605, "taxa_rateio": 0.05, "fatia_cargo": 0.2, "fc_detalhes": {"componentes": [{"nome_meta": "Faturamento da Linha", "peso": 0.15, "realizado": 85000.0, "meta": 100.0, "atingimento": 850.0, "atingimento_cap": 1.0, "componente_fc": 0.15}, {"nome_meta": "Conversão da Linha", "peso": 0.3, "realizado": 0.0, "meta": 100.0, "atingimento": 0.0, "atingimento_cap": 0.0, "componente_fc": 0.0}, {"nome_meta": "Rentabilidade", "peso": 0.2, "realizado": 0.255, "meta": 0.3330148556610093, "atingimento": 0.7657316052578024, "atingimento_cap": 0.7657316052578024, "componente_fc": 0.15314632105156048}, {"nome_meta": "Retenção de Clientes", "peso": 0.15, "realizado": 1.0, "meta": 0.0, "atingimento": 1.0, "atingimento_cap": 1.0, "componente_fc": 0.15}, {"nome_meta": "Meta Fornecedor 2", "peso": 0.1, "realizado": 0.0, "meta": 66.66666666666667, "atingimento": 0.0, "atingimento_cap": 0.0, "componente_fc": 0.0}], "fc_total": 0.4531463210515605}}], "total_valor": 50000.0, "soma_ponderada": 22657.316052578026, "fcmp_final": 0.4531463210515605}}</t>
+          <t>{"Alessandro Cappi": {"itens": [{"negocio": "SSO", "grupo": "Analisador Fixo", "subgrupo": "Falco", "tipo_mercadoria": "Produto", "valor": 50000.0, "taxa": 0.010000000000000002, "fc": 0.24008607120680028, "taxa_rateio": 0.05, "fatia_cargo": 0.2, "fc_detalhes": {"componentes": [{"nome_meta": "Faturamento da Linha", "peso": 0.15, "realizado": 412500.0, "meta": 0.0, "atingimento": 1.0, "atingimento_cap": 1.0, "componente_fc": 0.15}, {"nome_meta": "Conversão da Linha", "peso": 0.3, "realizado": 0.0, "meta": 0.0, "atingimento": 0.0, "atingimento_cap": 0.0, "componente_fc": 0.0}, {"nome_meta": "Rentabilidade", "peso": 0.2, "realizado": 0.15, "meta": 0.3330148556610093, "atingimento": 0.4504303560340014, "atingimento_cap": 0.4504303560340014, "componente_fc": 0.09008607120680029}, {"nome_meta": "Meta Fornecedor 2", "peso": 0.1, "realizado": 4370.56, "meta": 66.66666666666667, "atingimento": 65.5584, "atingimento_cap": 1.0, "componente_fc": 0.1}], "fc_total": 0.24008607120680028}}], "total_valor": 50000.0, "soma_ponderada": 12004.303560340015, "fcmp_final": 0.2400860712068003}}</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
@@ -2748,7 +3428,7 @@
         <v>3</v>
       </c>
       <c r="V9" s="7" t="n">
-        <v>45978.43176185185</v>
+        <v>45979.55425010416</v>
       </c>
       <c r="W9" t="inlineStr">
         <is>
@@ -2771,86 +3451,76 @@
         <v>8000</v>
       </c>
       <c r="C10" t="n">
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="D10" t="n">
-        <v>8000</v>
+        <v>0</v>
       </c>
       <c r="E10" t="n">
-        <v>8000</v>
+        <v>4000</v>
       </c>
       <c r="F10" t="n">
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="G10" t="n">
-        <v>0</v>
+        <v>40.00000000000001</v>
       </c>
       <c r="H10" t="n">
-        <v>63.19398202829279</v>
+        <v>0</v>
       </c>
       <c r="I10" t="n">
-        <v>63.19398202829279</v>
+        <v>40.00000000000001</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>FATURADO</t>
+          <t>ORCAMENTO</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>COMPLETO</t>
+          <t>PARCIAL</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>CALCULADO</t>
-        </is>
-      </c>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>08/2025</t>
+          <t>PENDENTE</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>{"André Caramello": 0.010000000000000002, "Alessandro Cappi": 0.010000000000000002}</t>
+          <t>{}</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>{"André Caramello": 0.3199623876768299, "Alessandro Cappi": 0.46996238767682985}</t>
+          <t>{}</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>{"André Caramello": {"itens": [{"negocio": "SSO", "grupo": "Analisador Fixo", "subgrupo": "Titan", "tipo_mercadoria": "Produto", "valor": 8000.0, "taxa": 0.010000000000000002, "fc": 0.3199623876768299, "taxa_rateio": 0.05, "fatia_cargo": 0.2, "fc_detalhes": {"componentes": [{"nome_meta": "Faturamento da Linha", "peso": 0.15, "realizado": 85000.0, "meta": 100.0, "atingimento": 850.0, "atingimento_cap": 1.0, "componente_fc": 0.15}, {"nome_meta": "Conversão da Linha", "peso": 0.3, "realizado": 0.0, "meta": 100.0, "atingimento": 0.0, "atingimento_cap": 0.0, "componente_fc": 0.0}, {"nome_meta": "Rentabilidade", "peso": 0.2, "realizado": 0.28300000000000003, "meta": 0.3330148556610093, "atingimento": 0.8498119383841494, "atingimento_cap": 0.8498119383841494, "componente_fc": 0.1699623876768299}, {"nome_meta": "Meta Fornecedor 2", "peso": 0.1, "realizado": 0.0, "meta": 66.66666666666667, "atingimento": 0.0, "atingimento_cap": 0.0, "componente_fc": 0.0}], "fc_total": 0.3199623876768299}}], "total_valor": 8000.0, "soma_ponderada": 80.00000000000001, "tcmp_final": 0.010000000000000002}, "Alessandro Cappi": {"itens": [{"negocio": "SSO", "grupo": "Analisador Fixo", "subgrupo": "Titan", "tipo_mercadoria": "Produto", "valor": 8000.0, "taxa": 0.010000000000000002, "fc": 0.46996238767682985, "taxa_rateio": 0.05, "fatia_cargo": 0.2, "fc_detalhes": {"componentes": [{"nome_meta": "Faturamento da Linha", "peso": 0.15, "realizado": 85000.0, "meta": 100.0, "atingimento": 850.0, "atingimento_cap": 1.0, "componente_fc": 0.15}, {"nome_meta": "Conversão da Linha", "peso": 0.3, "realizado": 0.0, "meta": 100.0, "atingimento": 0.0, "atingimento_cap": 0.0, "componente_fc": 0.0}, {"nome_meta": "Rentabilidade", "peso": 0.2, "realizado": 0.28300000000000003, "meta": 0.3330148556610093, "atingimento": 0.8498119383841494, "atingimento_cap": 0.8498119383841494, "componente_fc": 0.1699623876768299}, {"nome_meta": "Retenção de Clientes", "peso": 0.15, "realizado": 1.0, "meta": 0.0, "atingimento": 1.0, "atingimento_cap": 1.0, "componente_fc": 0.15}, {"nome_meta": "Meta Fornecedor 2", "peso": 0.1, "realizado": 0.0, "meta": 66.66666666666667, "atingimento": 0.0, "atingimento_cap": 0.0, "componente_fc": 0.0}], "fc_total": 0.46996238767682985}}], "total_valor": 8000.0, "soma_ponderada": 80.00000000000001, "tcmp_final": 0.010000000000000002}}</t>
+          <t>{}</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>{"André Caramello": {"itens": [{"negocio": "SSO", "grupo": "Analisador Fixo", "subgrupo": "Titan", "tipo_mercadoria": "Produto", "valor": 8000.0, "taxa": 0.010000000000000002, "fc": 0.3199623876768299, "taxa_rateio": 0.05, "fatia_cargo": 0.2, "fc_detalhes": {"componentes": [{"nome_meta": "Faturamento da Linha", "peso": 0.15, "realizado": 85000.0, "meta": 100.0, "atingimento": 850.0, "atingimento_cap": 1.0, "componente_fc": 0.15}, {"nome_meta": "Conversão da Linha", "peso": 0.3, "realizado": 0.0, "meta": 100.0, "atingimento": 0.0, "atingimento_cap": 0.0, "componente_fc": 0.0}, {"nome_meta": "Rentabilidade", "peso": 0.2, "realizado": 0.28300000000000003, "meta": 0.3330148556610093, "atingimento": 0.8498119383841494, "atingimento_cap": 0.8498119383841494, "componente_fc": 0.1699623876768299}, {"nome_meta": "Meta Fornecedor 2", "peso": 0.1, "realizado": 0.0, "meta": 66.66666666666667, "atingimento": 0.0, "atingimento_cap": 0.0, "componente_fc": 0.0}], "fc_total": 0.3199623876768299}}], "total_valor": 8000.0, "soma_ponderada": 2559.6991014146392, "fcmp_final": 0.3199623876768299}, "Alessandro Cappi": {"itens": [{"negocio": "SSO", "grupo": "Analisador Fixo", "subgrupo": "Titan", "tipo_mercadoria": "Produto", "valor": 8000.0, "taxa": 0.010000000000000002, "fc": 0.46996238767682985, "taxa_rateio": 0.05, "fatia_cargo": 0.2, "fc_detalhes": {"componentes": [{"nome_meta": "Faturamento da Linha", "peso": 0.15, "realizado": 85000.0, "meta": 100.0, "atingimento": 850.0, "atingimento_cap": 1.0, "componente_fc": 0.15}, {"nome_meta": "Conversão da Linha", "peso": 0.3, "realizado": 0.0, "meta": 100.0, "atingimento": 0.0, "atingimento_cap": 0.0, "componente_fc": 0.0}, {"nome_meta": "Rentabilidade", "peso": 0.2, "realizado": 0.28300000000000003, "meta": 0.3330148556610093, "atingimento": 0.8498119383841494, "atingimento_cap": 0.8498119383841494, "componente_fc": 0.1699623876768299}, {"nome_meta": "Retenção de Clientes", "peso": 0.15, "realizado": 1.0, "meta": 0.0, "atingimento": 1.0, "atingimento_cap": 1.0, "componente_fc": 0.15}, {"nome_meta": "Meta Fornecedor 2", "peso": 0.1, "realizado": 0.0, "meta": 66.66666666666667, "atingimento": 0.0, "atingimento_cap": 0.0, "componente_fc": 0.0}], "fc_total": 0.46996238767682985}}], "total_valor": 8000.0, "soma_ponderada": 3759.699101414639, "fcmp_final": 0.46996238767682985}}</t>
-        </is>
-      </c>
-      <c r="R10" t="inlineStr">
-        <is>
-          <t>André Caramello, Alessandro Cappi</t>
+          <t>{}</t>
         </is>
       </c>
       <c r="S10" s="7" t="n">
-        <v>45889</v>
+        <v>45887</v>
       </c>
       <c r="T10" s="7" t="n">
-        <v>45894</v>
+        <v>45887</v>
       </c>
       <c r="U10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="V10" s="7" t="n">
-        <v>45978.43176325232</v>
+        <v>45979.55425071759</v>
       </c>
       <c r="W10" t="inlineStr">
         <is>
-          <t>{}</t>
+          <t>{"Alessandro Cappi": 40.00000000000001}</t>
         </is>
       </c>
       <c r="X10" t="inlineStr">
@@ -2862,32 +3532,32 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>100010</t>
+          <t>200001</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>90000</v>
+        <v>15000</v>
       </c>
       <c r="C11" t="n">
-        <v>45000</v>
+        <v>7500</v>
       </c>
       <c r="D11" t="n">
         <v>0</v>
       </c>
       <c r="E11" t="n">
-        <v>45000</v>
+        <v>7500</v>
       </c>
       <c r="F11" t="n">
-        <v>45000</v>
+        <v>7500</v>
       </c>
       <c r="G11" t="n">
-        <v>450.0000000000001</v>
+        <v>75.00000000000001</v>
       </c>
       <c r="H11" t="n">
         <v>0</v>
       </c>
       <c r="I11" t="n">
-        <v>450.0000000000001</v>
+        <v>75.00000000000001</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
@@ -2925,23 +3595,1519 @@
         </is>
       </c>
       <c r="S11" s="7" t="n">
-        <v>45899</v>
+        <v>45875</v>
       </c>
       <c r="T11" s="7" t="n">
-        <v>45899</v>
+        <v>45875</v>
       </c>
       <c r="U11" t="n">
         <v>1</v>
       </c>
       <c r="V11" s="7" t="n">
-        <v>45978.43176497685</v>
+        <v>45979.55425115741</v>
       </c>
       <c r="W11" t="inlineStr">
         <is>
-          <t>{"Alessandro Cappi": 450.0000000000001}</t>
+          <t>{"Alessandro Cappi": 75.00000000000001}</t>
         </is>
       </c>
       <c r="X11" t="inlineStr">
+        <is>
+          <t>PENDENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>200002</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>15000</v>
+      </c>
+      <c r="C12" t="n">
+        <v>7500</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" t="n">
+        <v>7500</v>
+      </c>
+      <c r="F12" t="n">
+        <v>7500</v>
+      </c>
+      <c r="G12" t="n">
+        <v>75.00000000000001</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" t="n">
+        <v>75.00000000000001</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>ORCAMENTO</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>PARCIAL</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>PENDENTE</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="S12" s="7" t="n">
+        <v>45876</v>
+      </c>
+      <c r="T12" s="7" t="n">
+        <v>45876</v>
+      </c>
+      <c r="U12" t="n">
+        <v>1</v>
+      </c>
+      <c r="V12" s="7" t="n">
+        <v>45979.55425165509</v>
+      </c>
+      <c r="W12" t="inlineStr">
+        <is>
+          <t>{"Alessandro Cappi": 75.00000000000001}</t>
+        </is>
+      </c>
+      <c r="X12" t="inlineStr">
+        <is>
+          <t>PENDENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>200003</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>15000</v>
+      </c>
+      <c r="C13" t="n">
+        <v>7500</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" t="n">
+        <v>7500</v>
+      </c>
+      <c r="F13" t="n">
+        <v>7500</v>
+      </c>
+      <c r="G13" t="n">
+        <v>75.00000000000001</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" t="n">
+        <v>75.00000000000001</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>ORCAMENTO</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>PARCIAL</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>PENDENTE</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="S13" s="7" t="n">
+        <v>45877</v>
+      </c>
+      <c r="T13" s="7" t="n">
+        <v>45877</v>
+      </c>
+      <c r="U13" t="n">
+        <v>1</v>
+      </c>
+      <c r="V13" s="7" t="n">
+        <v>45979.55425223379</v>
+      </c>
+      <c r="W13" t="inlineStr">
+        <is>
+          <t>{"Alessandro Cappi": 75.00000000000001}</t>
+        </is>
+      </c>
+      <c r="X13" t="inlineStr">
+        <is>
+          <t>PENDENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>200004</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>15000</v>
+      </c>
+      <c r="C14" t="n">
+        <v>7500</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" t="n">
+        <v>7500</v>
+      </c>
+      <c r="F14" t="n">
+        <v>7500</v>
+      </c>
+      <c r="G14" t="n">
+        <v>75.00000000000001</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" t="n">
+        <v>75.00000000000001</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>ORCAMENTO</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>PARCIAL</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>PENDENTE</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="S14" s="7" t="n">
+        <v>45878</v>
+      </c>
+      <c r="T14" s="7" t="n">
+        <v>45878</v>
+      </c>
+      <c r="U14" t="n">
+        <v>1</v>
+      </c>
+      <c r="V14" s="7" t="n">
+        <v>45979.55425256945</v>
+      </c>
+      <c r="W14" t="inlineStr">
+        <is>
+          <t>{"Alessandro Cappi": 75.00000000000001}</t>
+        </is>
+      </c>
+      <c r="X14" t="inlineStr">
+        <is>
+          <t>PENDENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>200005</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>15000</v>
+      </c>
+      <c r="C15" t="n">
+        <v>7500</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" t="n">
+        <v>7500</v>
+      </c>
+      <c r="F15" t="n">
+        <v>7500</v>
+      </c>
+      <c r="G15" t="n">
+        <v>75.00000000000001</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" t="n">
+        <v>75.00000000000001</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>ORCAMENTO</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>PARCIAL</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>PENDENTE</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="S15" s="7" t="n">
+        <v>45879</v>
+      </c>
+      <c r="T15" s="7" t="n">
+        <v>45879</v>
+      </c>
+      <c r="U15" t="n">
+        <v>1</v>
+      </c>
+      <c r="V15" s="7" t="n">
+        <v>45979.55425290509</v>
+      </c>
+      <c r="W15" t="inlineStr">
+        <is>
+          <t>{"Alessandro Cappi": 75.00000000000001}</t>
+        </is>
+      </c>
+      <c r="X15" t="inlineStr">
+        <is>
+          <t>PENDENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>200006</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>15000</v>
+      </c>
+      <c r="C16" t="n">
+        <v>7500</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" t="n">
+        <v>7500</v>
+      </c>
+      <c r="F16" t="n">
+        <v>7500</v>
+      </c>
+      <c r="G16" t="n">
+        <v>75.00000000000001</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" t="n">
+        <v>75.00000000000001</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>ORCAMENTO</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>PARCIAL</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>PENDENTE</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="S16" s="7" t="n">
+        <v>45880</v>
+      </c>
+      <c r="T16" s="7" t="n">
+        <v>45880</v>
+      </c>
+      <c r="U16" t="n">
+        <v>1</v>
+      </c>
+      <c r="V16" s="7" t="n">
+        <v>45979.55425328704</v>
+      </c>
+      <c r="W16" t="inlineStr">
+        <is>
+          <t>{"Alessandro Cappi": 75.00000000000001}</t>
+        </is>
+      </c>
+      <c r="X16" t="inlineStr">
+        <is>
+          <t>PENDENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>200015</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>13500</v>
+      </c>
+      <c r="C17" t="n">
+        <v>6750</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" t="n">
+        <v>6750</v>
+      </c>
+      <c r="F17" t="n">
+        <v>6750</v>
+      </c>
+      <c r="G17" t="n">
+        <v>67.50000000000001</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" t="n">
+        <v>67.50000000000001</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>ORCAMENTO</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>PARCIAL</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>PENDENTE</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="S17" s="7" t="n">
+        <v>45889</v>
+      </c>
+      <c r="T17" s="7" t="n">
+        <v>45889</v>
+      </c>
+      <c r="U17" t="n">
+        <v>1</v>
+      </c>
+      <c r="V17" s="7" t="n">
+        <v>45979.55425371528</v>
+      </c>
+      <c r="W17" t="inlineStr">
+        <is>
+          <t>{"Alessandro Cappi": 67.50000000000001}</t>
+        </is>
+      </c>
+      <c r="X17" t="inlineStr">
+        <is>
+          <t>PENDENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>200018</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>13800</v>
+      </c>
+      <c r="C18" t="n">
+        <v>6900</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" t="n">
+        <v>6900</v>
+      </c>
+      <c r="F18" t="n">
+        <v>6900</v>
+      </c>
+      <c r="G18" t="n">
+        <v>69.00000000000001</v>
+      </c>
+      <c r="H18" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" t="n">
+        <v>69.00000000000001</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>ORCAMENTO</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>PARCIAL</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>PENDENTE</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="S18" s="7" t="n">
+        <v>45892</v>
+      </c>
+      <c r="T18" s="7" t="n">
+        <v>45892</v>
+      </c>
+      <c r="U18" t="n">
+        <v>1</v>
+      </c>
+      <c r="V18" s="7" t="n">
+        <v>45979.55425409722</v>
+      </c>
+      <c r="W18" t="inlineStr">
+        <is>
+          <t>{"Alessandro Cappi": 69.00000000000001}</t>
+        </is>
+      </c>
+      <c r="X18" t="inlineStr">
+        <is>
+          <t>PENDENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>200021</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>14100</v>
+      </c>
+      <c r="C19" t="n">
+        <v>7050</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" t="n">
+        <v>7050</v>
+      </c>
+      <c r="F19" t="n">
+        <v>7050</v>
+      </c>
+      <c r="G19" t="n">
+        <v>70.50000000000001</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" t="n">
+        <v>70.50000000000001</v>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>ORCAMENTO</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>PARCIAL</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>PENDENTE</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="S19" s="7" t="n">
+        <v>45875</v>
+      </c>
+      <c r="T19" s="7" t="n">
+        <v>45875</v>
+      </c>
+      <c r="U19" t="n">
+        <v>1</v>
+      </c>
+      <c r="V19" s="7" t="n">
+        <v>45979.55425443287</v>
+      </c>
+      <c r="W19" t="inlineStr">
+        <is>
+          <t>{"Alessandro Cappi": 70.50000000000001}</t>
+        </is>
+      </c>
+      <c r="X19" t="inlineStr">
+        <is>
+          <t>PENDENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>200024</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>14400</v>
+      </c>
+      <c r="C20" t="n">
+        <v>7200</v>
+      </c>
+      <c r="D20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" t="n">
+        <v>7200</v>
+      </c>
+      <c r="F20" t="n">
+        <v>7200</v>
+      </c>
+      <c r="G20" t="n">
+        <v>72.00000000000001</v>
+      </c>
+      <c r="H20" t="n">
+        <v>0</v>
+      </c>
+      <c r="I20" t="n">
+        <v>72.00000000000001</v>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>ORCAMENTO</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>PARCIAL</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>PENDENTE</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="S20" s="7" t="n">
+        <v>45878</v>
+      </c>
+      <c r="T20" s="7" t="n">
+        <v>45878</v>
+      </c>
+      <c r="U20" t="n">
+        <v>1</v>
+      </c>
+      <c r="V20" s="7" t="n">
+        <v>45979.55425482639</v>
+      </c>
+      <c r="W20" t="inlineStr">
+        <is>
+          <t>{"Alessandro Cappi": 72.00000000000001}</t>
+        </is>
+      </c>
+      <c r="X20" t="inlineStr">
+        <is>
+          <t>PENDENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>200027</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>14700</v>
+      </c>
+      <c r="C21" t="n">
+        <v>7350</v>
+      </c>
+      <c r="D21" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" t="n">
+        <v>7350</v>
+      </c>
+      <c r="F21" t="n">
+        <v>7350</v>
+      </c>
+      <c r="G21" t="n">
+        <v>73.50000000000001</v>
+      </c>
+      <c r="H21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I21" t="n">
+        <v>73.50000000000001</v>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>ORCAMENTO</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>PARCIAL</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>PENDENTE</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="S21" s="7" t="n">
+        <v>45881</v>
+      </c>
+      <c r="T21" s="7" t="n">
+        <v>45881</v>
+      </c>
+      <c r="U21" t="n">
+        <v>1</v>
+      </c>
+      <c r="V21" s="7" t="n">
+        <v>45979.55425518518</v>
+      </c>
+      <c r="W21" t="inlineStr">
+        <is>
+          <t>{"Alessandro Cappi": 73.50000000000001}</t>
+        </is>
+      </c>
+      <c r="X21" t="inlineStr">
+        <is>
+          <t>PENDENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>200030</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>15000</v>
+      </c>
+      <c r="C22" t="n">
+        <v>7500</v>
+      </c>
+      <c r="D22" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" t="n">
+        <v>7500</v>
+      </c>
+      <c r="F22" t="n">
+        <v>7500</v>
+      </c>
+      <c r="G22" t="n">
+        <v>75.00000000000001</v>
+      </c>
+      <c r="H22" t="n">
+        <v>0</v>
+      </c>
+      <c r="I22" t="n">
+        <v>75.00000000000001</v>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>ORCAMENTO</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>PARCIAL</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>PENDENTE</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="S22" s="7" t="n">
+        <v>45884</v>
+      </c>
+      <c r="T22" s="7" t="n">
+        <v>45884</v>
+      </c>
+      <c r="U22" t="n">
+        <v>1</v>
+      </c>
+      <c r="V22" s="7" t="n">
+        <v>45979.55425556713</v>
+      </c>
+      <c r="W22" t="inlineStr">
+        <is>
+          <t>{"Alessandro Cappi": 75.00000000000001}</t>
+        </is>
+      </c>
+      <c r="X22" t="inlineStr">
+        <is>
+          <t>PENDENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>200033</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>15300</v>
+      </c>
+      <c r="C23" t="n">
+        <v>7650</v>
+      </c>
+      <c r="D23" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" t="n">
+        <v>7650</v>
+      </c>
+      <c r="F23" t="n">
+        <v>7650</v>
+      </c>
+      <c r="G23" t="n">
+        <v>76.50000000000001</v>
+      </c>
+      <c r="H23" t="n">
+        <v>0</v>
+      </c>
+      <c r="I23" t="n">
+        <v>76.50000000000001</v>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>ORCAMENTO</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>PARCIAL</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>PENDENTE</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="S23" s="7" t="n">
+        <v>45887</v>
+      </c>
+      <c r="T23" s="7" t="n">
+        <v>45887</v>
+      </c>
+      <c r="U23" t="n">
+        <v>1</v>
+      </c>
+      <c r="V23" s="7" t="n">
+        <v>45979.5542559375</v>
+      </c>
+      <c r="W23" t="inlineStr">
+        <is>
+          <t>{"Alessandro Cappi": 76.50000000000001}</t>
+        </is>
+      </c>
+      <c r="X23" t="inlineStr">
+        <is>
+          <t>PENDENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>200036</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>15600</v>
+      </c>
+      <c r="C24" t="n">
+        <v>7800</v>
+      </c>
+      <c r="D24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" t="n">
+        <v>7800</v>
+      </c>
+      <c r="F24" t="n">
+        <v>7800</v>
+      </c>
+      <c r="G24" t="n">
+        <v>78.00000000000001</v>
+      </c>
+      <c r="H24" t="n">
+        <v>0</v>
+      </c>
+      <c r="I24" t="n">
+        <v>78.00000000000001</v>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>ORCAMENTO</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>PARCIAL</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>PENDENTE</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="S24" s="7" t="n">
+        <v>45890</v>
+      </c>
+      <c r="T24" s="7" t="n">
+        <v>45890</v>
+      </c>
+      <c r="U24" t="n">
+        <v>1</v>
+      </c>
+      <c r="V24" s="7" t="n">
+        <v>45979.55425629629</v>
+      </c>
+      <c r="W24" t="inlineStr">
+        <is>
+          <t>{"Alessandro Cappi": 78.00000000000001}</t>
+        </is>
+      </c>
+      <c r="X24" t="inlineStr">
+        <is>
+          <t>PENDENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>200039</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>15900</v>
+      </c>
+      <c r="C25" t="n">
+        <v>7950</v>
+      </c>
+      <c r="D25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" t="n">
+        <v>7950</v>
+      </c>
+      <c r="F25" t="n">
+        <v>7950</v>
+      </c>
+      <c r="G25" t="n">
+        <v>79.50000000000001</v>
+      </c>
+      <c r="H25" t="n">
+        <v>0</v>
+      </c>
+      <c r="I25" t="n">
+        <v>79.50000000000001</v>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>ORCAMENTO</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>PARCIAL</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>PENDENTE</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="S25" s="7" t="n">
+        <v>45893</v>
+      </c>
+      <c r="T25" s="7" t="n">
+        <v>45893</v>
+      </c>
+      <c r="U25" t="n">
+        <v>1</v>
+      </c>
+      <c r="V25" s="7" t="n">
+        <v>45979.55425664352</v>
+      </c>
+      <c r="W25" t="inlineStr">
+        <is>
+          <t>{"Alessandro Cappi": 79.50000000000001}</t>
+        </is>
+      </c>
+      <c r="X25" t="inlineStr">
+        <is>
+          <t>PENDENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>200042</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>16200</v>
+      </c>
+      <c r="C26" t="n">
+        <v>8100</v>
+      </c>
+      <c r="D26" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" t="n">
+        <v>8100</v>
+      </c>
+      <c r="F26" t="n">
+        <v>8100</v>
+      </c>
+      <c r="G26" t="n">
+        <v>81.00000000000001</v>
+      </c>
+      <c r="H26" t="n">
+        <v>0</v>
+      </c>
+      <c r="I26" t="n">
+        <v>81.00000000000001</v>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>ORCAMENTO</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>PARCIAL</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>PENDENTE</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="S26" s="7" t="n">
+        <v>45876</v>
+      </c>
+      <c r="T26" s="7" t="n">
+        <v>45876</v>
+      </c>
+      <c r="U26" t="n">
+        <v>1</v>
+      </c>
+      <c r="V26" s="7" t="n">
+        <v>45979.55425697917</v>
+      </c>
+      <c r="W26" t="inlineStr">
+        <is>
+          <t>{"Alessandro Cappi": 81.00000000000001}</t>
+        </is>
+      </c>
+      <c r="X26" t="inlineStr">
+        <is>
+          <t>PENDENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>200045</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>16500</v>
+      </c>
+      <c r="C27" t="n">
+        <v>8250</v>
+      </c>
+      <c r="D27" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" t="n">
+        <v>8250</v>
+      </c>
+      <c r="F27" t="n">
+        <v>8250</v>
+      </c>
+      <c r="G27" t="n">
+        <v>82.50000000000001</v>
+      </c>
+      <c r="H27" t="n">
+        <v>0</v>
+      </c>
+      <c r="I27" t="n">
+        <v>82.50000000000001</v>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>ORCAMENTO</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>PARCIAL</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>PENDENTE</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="S27" s="7" t="n">
+        <v>45879</v>
+      </c>
+      <c r="T27" s="7" t="n">
+        <v>45879</v>
+      </c>
+      <c r="U27" t="n">
+        <v>1</v>
+      </c>
+      <c r="V27" s="7" t="n">
+        <v>45979.55425741898</v>
+      </c>
+      <c r="W27" t="inlineStr">
+        <is>
+          <t>{"Alessandro Cappi": 82.50000000000001}</t>
+        </is>
+      </c>
+      <c r="X27" t="inlineStr">
+        <is>
+          <t>PENDENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>200048</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>16800</v>
+      </c>
+      <c r="C28" t="n">
+        <v>8400</v>
+      </c>
+      <c r="D28" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" t="n">
+        <v>8400</v>
+      </c>
+      <c r="F28" t="n">
+        <v>8400</v>
+      </c>
+      <c r="G28" t="n">
+        <v>84.00000000000001</v>
+      </c>
+      <c r="H28" t="n">
+        <v>0</v>
+      </c>
+      <c r="I28" t="n">
+        <v>84.00000000000001</v>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>ORCAMENTO</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>PARCIAL</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>PENDENTE</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="S28" s="7" t="n">
+        <v>45882</v>
+      </c>
+      <c r="T28" s="7" t="n">
+        <v>45882</v>
+      </c>
+      <c r="U28" t="n">
+        <v>1</v>
+      </c>
+      <c r="V28" s="7" t="n">
+        <v>45979.55425773148</v>
+      </c>
+      <c r="W28" t="inlineStr">
+        <is>
+          <t>{"Alessandro Cappi": 84.00000000000001}</t>
+        </is>
+      </c>
+      <c r="X28" t="inlineStr">
         <is>
           <t>PENDENTE</t>
         </is>
@@ -2958,14 +5124,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="50" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
     <col width="7" customWidth="1" min="4" max="4"/>
-    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2995,52 +5161,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>XYZ999</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>XYZ999</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Documento muito curto (menos de 5 dígitos): XYZ999</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>1000</v>
-      </c>
-      <c r="E2" s="7" t="n">
-        <v>45884</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>COT</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>COT</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>COT sem sufixo numérico válido: COT</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>500</v>
-      </c>
-      <c r="E3" s="7" t="n">
-        <v>45885</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
CORREÇÃO CROSS-SELLING UTILIZANDO FALLBACK DE 1%
</commit_message>
<xml_diff>
--- a/Comissoes_Recebimento_08_2025.xlsx
+++ b/Comissoes_Recebimento_08_2025.xlsx
@@ -39,7 +39,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -64,12 +64,6 @@
         <bgColor rgb="00F1F8E9"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFF3E0"/>
-        <bgColor rgb="00FFF3E0"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -89,7 +83,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
@@ -100,7 +94,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -2283,13 +2276,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
     <col width="6" customWidth="1" min="3" max="3"/>
-    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="6" customWidth="1" min="4" max="4"/>
     <col width="25" customWidth="1" min="5" max="5"/>
     <col width="26" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
@@ -2341,41 +2334,6 @@
       <c r="I1" s="3" t="inlineStr">
         <is>
           <t>mes_faturamento</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="6" t="inlineStr">
-        <is>
-          <t>100002</t>
-        </is>
-      </c>
-      <c r="B2" s="6" t="inlineStr">
-        <is>
-          <t>Alessandro Cappi</t>
-        </is>
-      </c>
-      <c r="C2" s="6" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="D2" s="6" t="n">
-        <v>0.52134</v>
-      </c>
-      <c r="E2" s="6" t="n">
-        <v>60</v>
-      </c>
-      <c r="F2" s="6" t="n">
-        <v>31.2804</v>
-      </c>
-      <c r="G2" s="6" t="n">
-        <v>-0.47866</v>
-      </c>
-      <c r="H2" s="6" t="n">
-        <v>-28.7196</v>
-      </c>
-      <c r="I2" s="6" t="inlineStr">
-        <is>
-          <t>08/2025</t>
         </is>
       </c>
     </row>
@@ -2557,25 +2515,25 @@
         <v>8000</v>
       </c>
       <c r="C2" t="n">
-        <v>4000</v>
+        <v>72000</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>4000</v>
+        <v>72000</v>
       </c>
       <c r="F2" t="n">
-        <v>4000</v>
+        <v>-64000</v>
       </c>
       <c r="G2" t="n">
-        <v>40.00000000000001</v>
+        <v>720</v>
       </c>
       <c r="H2" t="n">
         <v>0</v>
       </c>
       <c r="I2" t="n">
-        <v>40.00000000000001</v>
+        <v>720</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -2584,7 +2542,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>PARCIAL</t>
+          <t>COMPLETO</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -2612,21 +2570,21 @@
           <t>{}</t>
         </is>
       </c>
-      <c r="S2" s="7" t="n">
+      <c r="S2" s="6" t="n">
         <v>45879</v>
       </c>
-      <c r="T2" s="7" t="n">
+      <c r="T2" s="6" t="n">
         <v>45879</v>
       </c>
       <c r="U2" t="n">
-        <v>1</v>
-      </c>
-      <c r="V2" s="7" t="n">
-        <v>45987.69724752315</v>
+        <v>18</v>
+      </c>
+      <c r="V2" s="6" t="n">
+        <v>45987.74509543982</v>
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>{"Alessandro Cappi": 40.00000000000001}</t>
+          <t>{"Alessandro Cappi": 720.0000000000001}</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
@@ -2645,25 +2603,25 @@
         <v>12000</v>
       </c>
       <c r="C3" t="n">
-        <v>6000</v>
+        <v>108000</v>
       </c>
       <c r="D3" t="n">
-        <v>6000</v>
+        <v>108000</v>
       </c>
       <c r="E3" t="n">
-        <v>12000</v>
+        <v>216000</v>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>-204000</v>
       </c>
       <c r="G3" t="n">
-        <v>60.00000000000001</v>
+        <v>1080</v>
       </c>
       <c r="H3" t="n">
-        <v>31.2804</v>
+        <v>563.0472</v>
       </c>
       <c r="I3" t="n">
-        <v>91.28040000000001</v>
+        <v>1643.0472</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
@@ -2710,21 +2668,21 @@
           <t>Alessandro Cappi</t>
         </is>
       </c>
-      <c r="S3" s="7" t="n">
+      <c r="S3" s="6" t="n">
         <v>45874</v>
       </c>
-      <c r="T3" s="7" t="n">
+      <c r="T3" s="6" t="n">
         <v>45897</v>
       </c>
       <c r="U3" t="n">
-        <v>2</v>
-      </c>
-      <c r="V3" s="7" t="n">
-        <v>45987.69727850694</v>
+        <v>36</v>
+      </c>
+      <c r="V3" s="6" t="n">
+        <v>45987.74509609953</v>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>{"Alessandro Cappi": 60.000000000000014}</t>
+          <t>{"Alessandro Cappi": 1080.0000000000002}</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
@@ -2743,25 +2701,25 @@
         <v>15000</v>
       </c>
       <c r="C4" t="n">
-        <v>7500</v>
+        <v>135000</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>7500</v>
+        <v>135000</v>
       </c>
       <c r="F4" t="n">
-        <v>7500</v>
+        <v>-120000</v>
       </c>
       <c r="G4" t="n">
-        <v>75.00000000000001</v>
+        <v>1350</v>
       </c>
       <c r="H4" t="n">
         <v>0</v>
       </c>
       <c r="I4" t="n">
-        <v>75.00000000000001</v>
+        <v>1350</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
@@ -2770,7 +2728,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>PARCIAL</t>
+          <t>COMPLETO</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -2798,21 +2756,21 @@
           <t>{}</t>
         </is>
       </c>
-      <c r="S4" s="7" t="n">
+      <c r="S4" s="6" t="n">
         <v>45881</v>
       </c>
-      <c r="T4" s="7" t="n">
+      <c r="T4" s="6" t="n">
         <v>45881</v>
       </c>
       <c r="U4" t="n">
-        <v>1</v>
-      </c>
-      <c r="V4" s="7" t="n">
-        <v>45987.697250625</v>
+        <v>18</v>
+      </c>
+      <c r="V4" s="6" t="n">
+        <v>45987.74509650463</v>
       </c>
       <c r="W4" t="inlineStr">
         <is>
-          <t>{"Alessandro Cappi": 75.00000000000001}</t>
+          <t>{"Alessandro Cappi": 1350.0000000000002}</t>
         </is>
       </c>
       <c r="X4" t="inlineStr">
@@ -2831,25 +2789,25 @@
         <v>18000</v>
       </c>
       <c r="C5" t="n">
-        <v>11000</v>
+        <v>198000</v>
       </c>
       <c r="D5" t="n">
         <v>0</v>
       </c>
       <c r="E5" t="n">
-        <v>11000</v>
+        <v>198000</v>
       </c>
       <c r="F5" t="n">
-        <v>7000</v>
+        <v>-180000</v>
       </c>
       <c r="G5" t="n">
-        <v>110</v>
+        <v>1980</v>
       </c>
       <c r="H5" t="n">
         <v>0</v>
       </c>
       <c r="I5" t="n">
-        <v>110</v>
+        <v>1980</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
@@ -2858,7 +2816,7 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>PARCIAL</t>
+          <t>COMPLETO</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -2886,21 +2844,21 @@
           <t>{}</t>
         </is>
       </c>
-      <c r="S5" s="7" t="n">
+      <c r="S5" s="6" t="n">
         <v>45877</v>
       </c>
-      <c r="T5" s="7" t="n">
+      <c r="T5" s="6" t="n">
         <v>45884</v>
       </c>
       <c r="U5" t="n">
-        <v>2</v>
-      </c>
-      <c r="V5" s="7" t="n">
-        <v>45987.69725278935</v>
+        <v>36</v>
+      </c>
+      <c r="V5" s="6" t="n">
+        <v>45987.74509731482</v>
       </c>
       <c r="W5" t="inlineStr">
         <is>
-          <t>{"Alessandro Cappi": 110.00000000000003}</t>
+          <t>{"Alessandro Cappi": 1980.0000000000002}</t>
         </is>
       </c>
       <c r="X5" t="inlineStr">
@@ -2922,22 +2880,22 @@
         <v>0</v>
       </c>
       <c r="D6" t="n">
-        <v>10000</v>
+        <v>180000</v>
       </c>
       <c r="E6" t="n">
-        <v>10000</v>
+        <v>180000</v>
       </c>
       <c r="F6" t="n">
-        <v>0</v>
+        <v>-170000</v>
       </c>
       <c r="G6" t="n">
         <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>56.934</v>
+        <v>1024.812</v>
       </c>
       <c r="I6" t="n">
-        <v>56.934</v>
+        <v>1024.812</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
@@ -2984,17 +2942,17 @@
           <t>Alessandro Cappi</t>
         </is>
       </c>
-      <c r="S6" s="7" t="n">
+      <c r="S6" s="6" t="n">
         <v>45891</v>
       </c>
-      <c r="T6" s="7" t="n">
+      <c r="T6" s="6" t="n">
         <v>45898</v>
       </c>
       <c r="U6" t="n">
-        <v>2</v>
-      </c>
-      <c r="V6" s="7" t="n">
-        <v>45987.69725376157</v>
+        <v>36</v>
+      </c>
+      <c r="V6" s="6" t="n">
+        <v>45987.7450975</v>
       </c>
       <c r="W6" t="inlineStr">
         <is>
@@ -3017,25 +2975,25 @@
         <v>22000</v>
       </c>
       <c r="C7" t="n">
-        <v>11000</v>
+        <v>198000</v>
       </c>
       <c r="D7" t="n">
         <v>0</v>
       </c>
       <c r="E7" t="n">
-        <v>11000</v>
+        <v>198000</v>
       </c>
       <c r="F7" t="n">
-        <v>11000</v>
+        <v>-176000</v>
       </c>
       <c r="G7" t="n">
-        <v>110</v>
+        <v>1980</v>
       </c>
       <c r="H7" t="n">
         <v>0</v>
       </c>
       <c r="I7" t="n">
-        <v>110</v>
+        <v>1980</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
@@ -3044,7 +3002,7 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>PARCIAL</t>
+          <t>COMPLETO</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -3072,21 +3030,21 @@
           <t>{}</t>
         </is>
       </c>
-      <c r="S7" s="7" t="n">
+      <c r="S7" s="6" t="n">
         <v>45889</v>
       </c>
-      <c r="T7" s="7" t="n">
+      <c r="T7" s="6" t="n">
         <v>45889</v>
       </c>
       <c r="U7" t="n">
-        <v>1</v>
-      </c>
-      <c r="V7" s="7" t="n">
-        <v>45987.69725518519</v>
+        <v>18</v>
+      </c>
+      <c r="V7" s="6" t="n">
+        <v>45987.74509832176</v>
       </c>
       <c r="W7" t="inlineStr">
         <is>
-          <t>{"Alessandro Cappi": 110.00000000000003}</t>
+          <t>{"Alessandro Cappi": 1980.0000000000002}</t>
         </is>
       </c>
       <c r="X7" t="inlineStr">
@@ -3105,25 +3063,25 @@
         <v>105000</v>
       </c>
       <c r="C8" t="n">
-        <v>52500</v>
+        <v>945000</v>
       </c>
       <c r="D8" t="n">
         <v>0</v>
       </c>
       <c r="E8" t="n">
-        <v>52500</v>
+        <v>945000</v>
       </c>
       <c r="F8" t="n">
-        <v>52500</v>
+        <v>-840000</v>
       </c>
       <c r="G8" t="n">
-        <v>525.0000000000001</v>
+        <v>9450</v>
       </c>
       <c r="H8" t="n">
         <v>0</v>
       </c>
       <c r="I8" t="n">
-        <v>525.0000000000001</v>
+        <v>9450</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
@@ -3132,7 +3090,7 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>PARCIAL</t>
+          <t>COMPLETO</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -3160,21 +3118,21 @@
           <t>{}</t>
         </is>
       </c>
-      <c r="S8" s="7" t="n">
+      <c r="S8" s="6" t="n">
         <v>45894</v>
       </c>
-      <c r="T8" s="7" t="n">
+      <c r="T8" s="6" t="n">
         <v>45894</v>
       </c>
       <c r="U8" t="n">
-        <v>1</v>
-      </c>
-      <c r="V8" s="7" t="n">
-        <v>45987.69725615741</v>
+        <v>18</v>
+      </c>
+      <c r="V8" s="6" t="n">
+        <v>45987.74509914352</v>
       </c>
       <c r="W8" t="inlineStr">
         <is>
-          <t>{"Alessandro Cappi": 525.0000000000001}</t>
+          <t>{"Alessandro Cappi": 9450.000000000002}</t>
         </is>
       </c>
       <c r="X8" t="inlineStr">
@@ -3196,22 +3154,22 @@
         <v>0</v>
       </c>
       <c r="D9" t="n">
-        <v>16000</v>
+        <v>288000</v>
       </c>
       <c r="E9" t="n">
-        <v>16000</v>
+        <v>288000</v>
       </c>
       <c r="F9" t="n">
-        <v>0</v>
+        <v>-272000</v>
       </c>
       <c r="G9" t="n">
         <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>83.4144</v>
+        <v>1501.4592</v>
       </c>
       <c r="I9" t="n">
-        <v>83.4144</v>
+        <v>1501.4592</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
@@ -3258,17 +3216,17 @@
           <t>Alessandro Cappi</t>
         </is>
       </c>
-      <c r="S9" s="7" t="n">
+      <c r="S9" s="6" t="n">
         <v>45887</v>
       </c>
-      <c r="T9" s="7" t="n">
+      <c r="T9" s="6" t="n">
         <v>45897</v>
       </c>
       <c r="U9" t="n">
-        <v>3</v>
-      </c>
-      <c r="V9" s="7" t="n">
-        <v>45987.69725738426</v>
+        <v>54</v>
+      </c>
+      <c r="V9" s="6" t="n">
+        <v>45987.74509935185</v>
       </c>
       <c r="W9" t="inlineStr">
         <is>
@@ -3291,25 +3249,25 @@
         <v>6000</v>
       </c>
       <c r="C10" t="n">
-        <v>3000</v>
+        <v>54000</v>
       </c>
       <c r="D10" t="n">
         <v>0</v>
       </c>
       <c r="E10" t="n">
-        <v>3000</v>
+        <v>54000</v>
       </c>
       <c r="F10" t="n">
-        <v>3000</v>
+        <v>-48000</v>
       </c>
       <c r="G10" t="n">
-        <v>30.00000000000001</v>
+        <v>540</v>
       </c>
       <c r="H10" t="n">
         <v>0</v>
       </c>
       <c r="I10" t="n">
-        <v>30.00000000000001</v>
+        <v>540</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
@@ -3318,7 +3276,7 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>PARCIAL</t>
+          <t>COMPLETO</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -3346,21 +3304,21 @@
           <t>{}</t>
         </is>
       </c>
-      <c r="S10" s="7" t="n">
+      <c r="S10" s="6" t="n">
         <v>45887</v>
       </c>
-      <c r="T10" s="7" t="n">
+      <c r="T10" s="6" t="n">
         <v>45887</v>
       </c>
       <c r="U10" t="n">
-        <v>1</v>
-      </c>
-      <c r="V10" s="7" t="n">
-        <v>45987.69725975695</v>
+        <v>18</v>
+      </c>
+      <c r="V10" s="6" t="n">
+        <v>45987.74509976852</v>
       </c>
       <c r="W10" t="inlineStr">
         <is>
-          <t>{"Alessandro Cappi": 30.000000000000007}</t>
+          <t>{"Alessandro Cappi": 540.0000000000001}</t>
         </is>
       </c>
       <c r="X10" t="inlineStr">
@@ -3379,25 +3337,25 @@
         <v>14000</v>
       </c>
       <c r="C11" t="n">
-        <v>7000</v>
+        <v>126000</v>
       </c>
       <c r="D11" t="n">
         <v>0</v>
       </c>
       <c r="E11" t="n">
-        <v>7000</v>
+        <v>126000</v>
       </c>
       <c r="F11" t="n">
-        <v>7000</v>
+        <v>-112000</v>
       </c>
       <c r="G11" t="n">
-        <v>70.00000000000001</v>
+        <v>1260</v>
       </c>
       <c r="H11" t="n">
         <v>0</v>
       </c>
       <c r="I11" t="n">
-        <v>70.00000000000001</v>
+        <v>1260</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
@@ -3406,7 +3364,7 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>PARCIAL</t>
+          <t>COMPLETO</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -3434,21 +3392,21 @@
           <t>{}</t>
         </is>
       </c>
-      <c r="S11" s="7" t="n">
+      <c r="S11" s="6" t="n">
         <v>45875</v>
       </c>
-      <c r="T11" s="7" t="n">
+      <c r="T11" s="6" t="n">
         <v>45875</v>
       </c>
       <c r="U11" t="n">
-        <v>1</v>
-      </c>
-      <c r="V11" s="7" t="n">
-        <v>45987.69726092592</v>
+        <v>18</v>
+      </c>
+      <c r="V11" s="6" t="n">
+        <v>45987.74510023148</v>
       </c>
       <c r="W11" t="inlineStr">
         <is>
-          <t>{"Alessandro Cappi": 70.00000000000001}</t>
+          <t>{"Alessandro Cappi": 1260.0000000000002}</t>
         </is>
       </c>
       <c r="X11" t="inlineStr">
@@ -3467,25 +3425,25 @@
         <v>16000</v>
       </c>
       <c r="C12" t="n">
-        <v>8000</v>
+        <v>144000</v>
       </c>
       <c r="D12" t="n">
         <v>0</v>
       </c>
       <c r="E12" t="n">
-        <v>8000</v>
+        <v>144000</v>
       </c>
       <c r="F12" t="n">
-        <v>8000</v>
+        <v>-128000</v>
       </c>
       <c r="G12" t="n">
-        <v>80.00000000000001</v>
+        <v>1440</v>
       </c>
       <c r="H12" t="n">
         <v>0</v>
       </c>
       <c r="I12" t="n">
-        <v>80.00000000000001</v>
+        <v>1440</v>
       </c>
       <c r="J12" t="inlineStr">
         <is>
@@ -3494,7 +3452,7 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>PARCIAL</t>
+          <t>COMPLETO</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -3522,21 +3480,21 @@
           <t>{}</t>
         </is>
       </c>
-      <c r="S12" s="7" t="n">
+      <c r="S12" s="6" t="n">
         <v>45876</v>
       </c>
-      <c r="T12" s="7" t="n">
+      <c r="T12" s="6" t="n">
         <v>45876</v>
       </c>
       <c r="U12" t="n">
-        <v>1</v>
-      </c>
-      <c r="V12" s="7" t="n">
-        <v>45987.69726171296</v>
+        <v>18</v>
+      </c>
+      <c r="V12" s="6" t="n">
+        <v>45987.74510061343</v>
       </c>
       <c r="W12" t="inlineStr">
         <is>
-          <t>{"Alessandro Cappi": 80.00000000000001}</t>
+          <t>{"Alessandro Cappi": 1440.0000000000002}</t>
         </is>
       </c>
       <c r="X12" t="inlineStr">
@@ -3555,25 +3513,25 @@
         <v>18000</v>
       </c>
       <c r="C13" t="n">
-        <v>9000</v>
+        <v>162000</v>
       </c>
       <c r="D13" t="n">
         <v>0</v>
       </c>
       <c r="E13" t="n">
-        <v>9000</v>
+        <v>162000</v>
       </c>
       <c r="F13" t="n">
-        <v>9000</v>
+        <v>-144000</v>
       </c>
       <c r="G13" t="n">
-        <v>90.00000000000001</v>
+        <v>1620</v>
       </c>
       <c r="H13" t="n">
         <v>0</v>
       </c>
       <c r="I13" t="n">
-        <v>90.00000000000001</v>
+        <v>1620</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
@@ -3582,7 +3540,7 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>PARCIAL</t>
+          <t>COMPLETO</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -3610,21 +3568,21 @@
           <t>{}</t>
         </is>
       </c>
-      <c r="S13" s="7" t="n">
+      <c r="S13" s="6" t="n">
         <v>45877</v>
       </c>
-      <c r="T13" s="7" t="n">
+      <c r="T13" s="6" t="n">
         <v>45877</v>
       </c>
       <c r="U13" t="n">
-        <v>1</v>
-      </c>
-      <c r="V13" s="7" t="n">
-        <v>45987.69726258102</v>
+        <v>18</v>
+      </c>
+      <c r="V13" s="6" t="n">
+        <v>45987.74510100694</v>
       </c>
       <c r="W13" t="inlineStr">
         <is>
-          <t>{"Alessandro Cappi": 90.00000000000001}</t>
+          <t>{"Alessandro Cappi": 1620.0000000000002}</t>
         </is>
       </c>
       <c r="X13" t="inlineStr">
@@ -3643,25 +3601,25 @@
         <v>20000</v>
       </c>
       <c r="C14" t="n">
-        <v>10000</v>
+        <v>180000</v>
       </c>
       <c r="D14" t="n">
         <v>0</v>
       </c>
       <c r="E14" t="n">
-        <v>10000</v>
+        <v>180000</v>
       </c>
       <c r="F14" t="n">
-        <v>10000</v>
+        <v>-160000</v>
       </c>
       <c r="G14" t="n">
-        <v>100</v>
+        <v>1800</v>
       </c>
       <c r="H14" t="n">
         <v>0</v>
       </c>
       <c r="I14" t="n">
-        <v>100</v>
+        <v>1800</v>
       </c>
       <c r="J14" t="inlineStr">
         <is>
@@ -3670,7 +3628,7 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>PARCIAL</t>
+          <t>COMPLETO</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -3698,21 +3656,21 @@
           <t>{}</t>
         </is>
       </c>
-      <c r="S14" s="7" t="n">
+      <c r="S14" s="6" t="n">
         <v>45878</v>
       </c>
-      <c r="T14" s="7" t="n">
+      <c r="T14" s="6" t="n">
         <v>45878</v>
       </c>
       <c r="U14" t="n">
-        <v>1</v>
-      </c>
-      <c r="V14" s="7" t="n">
-        <v>45987.6972633912</v>
+        <v>18</v>
+      </c>
+      <c r="V14" s="6" t="n">
+        <v>45987.74510138889</v>
       </c>
       <c r="W14" t="inlineStr">
         <is>
-          <t>{"Alessandro Cappi": 100.00000000000001}</t>
+          <t>{"Alessandro Cappi": 1800.0000000000002}</t>
         </is>
       </c>
       <c r="X14" t="inlineStr">
@@ -3731,25 +3689,25 @@
         <v>22000</v>
       </c>
       <c r="C15" t="n">
-        <v>11000</v>
+        <v>198000</v>
       </c>
       <c r="D15" t="n">
         <v>0</v>
       </c>
       <c r="E15" t="n">
-        <v>11000</v>
+        <v>198000</v>
       </c>
       <c r="F15" t="n">
-        <v>11000</v>
+        <v>-176000</v>
       </c>
       <c r="G15" t="n">
-        <v>110</v>
+        <v>1980</v>
       </c>
       <c r="H15" t="n">
         <v>0</v>
       </c>
       <c r="I15" t="n">
-        <v>110</v>
+        <v>1980</v>
       </c>
       <c r="J15" t="inlineStr">
         <is>
@@ -3758,7 +3716,7 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>PARCIAL</t>
+          <t>COMPLETO</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
@@ -3786,21 +3744,21 @@
           <t>{}</t>
         </is>
       </c>
-      <c r="S15" s="7" t="n">
+      <c r="S15" s="6" t="n">
         <v>45879</v>
       </c>
-      <c r="T15" s="7" t="n">
+      <c r="T15" s="6" t="n">
         <v>45879</v>
       </c>
       <c r="U15" t="n">
-        <v>1</v>
-      </c>
-      <c r="V15" s="7" t="n">
-        <v>45987.69726424768</v>
+        <v>18</v>
+      </c>
+      <c r="V15" s="6" t="n">
+        <v>45987.74510181713</v>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>{"Alessandro Cappi": 110.00000000000003}</t>
+          <t>{"Alessandro Cappi": 1980.0000000000002}</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
@@ -3819,25 +3777,25 @@
         <v>24000</v>
       </c>
       <c r="C16" t="n">
-        <v>12000</v>
+        <v>216000</v>
       </c>
       <c r="D16" t="n">
         <v>0</v>
       </c>
       <c r="E16" t="n">
-        <v>12000</v>
+        <v>216000</v>
       </c>
       <c r="F16" t="n">
-        <v>12000</v>
+        <v>-192000</v>
       </c>
       <c r="G16" t="n">
-        <v>120</v>
+        <v>2160</v>
       </c>
       <c r="H16" t="n">
         <v>0</v>
       </c>
       <c r="I16" t="n">
-        <v>120</v>
+        <v>2160</v>
       </c>
       <c r="J16" t="inlineStr">
         <is>
@@ -3846,7 +3804,7 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>PARCIAL</t>
+          <t>COMPLETO</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -3874,21 +3832,21 @@
           <t>{}</t>
         </is>
       </c>
-      <c r="S16" s="7" t="n">
+      <c r="S16" s="6" t="n">
         <v>45880</v>
       </c>
-      <c r="T16" s="7" t="n">
+      <c r="T16" s="6" t="n">
         <v>45880</v>
       </c>
       <c r="U16" t="n">
-        <v>1</v>
-      </c>
-      <c r="V16" s="7" t="n">
-        <v>45987.69726576389</v>
+        <v>18</v>
+      </c>
+      <c r="V16" s="6" t="n">
+        <v>45987.74510221065</v>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>{"Alessandro Cappi": 120.00000000000003}</t>
+          <t>{"Alessandro Cappi": 2160.0000000000005}</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
@@ -3907,25 +3865,25 @@
         <v>5600</v>
       </c>
       <c r="C17" t="n">
-        <v>2800</v>
+        <v>50400</v>
       </c>
       <c r="D17" t="n">
         <v>0</v>
       </c>
       <c r="E17" t="n">
-        <v>2800</v>
+        <v>50400</v>
       </c>
       <c r="F17" t="n">
-        <v>2800</v>
+        <v>-44800</v>
       </c>
       <c r="G17" t="n">
-        <v>28.00000000000001</v>
+        <v>504</v>
       </c>
       <c r="H17" t="n">
         <v>0</v>
       </c>
       <c r="I17" t="n">
-        <v>28.00000000000001</v>
+        <v>504</v>
       </c>
       <c r="J17" t="inlineStr">
         <is>
@@ -3934,7 +3892,7 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>PARCIAL</t>
+          <t>COMPLETO</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
@@ -3962,21 +3920,21 @@
           <t>{}</t>
         </is>
       </c>
-      <c r="S17" s="7" t="n">
+      <c r="S17" s="6" t="n">
         <v>45889</v>
       </c>
-      <c r="T17" s="7" t="n">
+      <c r="T17" s="6" t="n">
         <v>45889</v>
       </c>
       <c r="U17" t="n">
-        <v>1</v>
-      </c>
-      <c r="V17" s="7" t="n">
-        <v>45987.69726666667</v>
+        <v>18</v>
+      </c>
+      <c r="V17" s="6" t="n">
+        <v>45987.74510261574</v>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>{"Alessandro Cappi": 28.000000000000007}</t>
+          <t>{"Alessandro Cappi": 504.00000000000006}</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
@@ -3995,25 +3953,25 @@
         <v>6500</v>
       </c>
       <c r="C18" t="n">
-        <v>3250</v>
+        <v>58500</v>
       </c>
       <c r="D18" t="n">
         <v>0</v>
       </c>
       <c r="E18" t="n">
-        <v>3250</v>
+        <v>58500</v>
       </c>
       <c r="F18" t="n">
-        <v>3250</v>
+        <v>-52000</v>
       </c>
       <c r="G18" t="n">
-        <v>32.50000000000001</v>
+        <v>585</v>
       </c>
       <c r="H18" t="n">
         <v>0</v>
       </c>
       <c r="I18" t="n">
-        <v>32.50000000000001</v>
+        <v>585</v>
       </c>
       <c r="J18" t="inlineStr">
         <is>
@@ -4022,7 +3980,7 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>PARCIAL</t>
+          <t>COMPLETO</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
@@ -4050,21 +4008,21 @@
           <t>{}</t>
         </is>
       </c>
-      <c r="S18" s="7" t="n">
+      <c r="S18" s="6" t="n">
         <v>45892</v>
       </c>
-      <c r="T18" s="7" t="n">
+      <c r="T18" s="6" t="n">
         <v>45892</v>
       </c>
       <c r="U18" t="n">
-        <v>1</v>
-      </c>
-      <c r="V18" s="7" t="n">
-        <v>45987.69726784722</v>
+        <v>18</v>
+      </c>
+      <c r="V18" s="6" t="n">
+        <v>45987.74510302083</v>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>{"Alessandro Cappi": 32.50000000000001}</t>
+          <t>{"Alessandro Cappi": 585.0000000000001}</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
@@ -4083,25 +4041,25 @@
         <v>7400</v>
       </c>
       <c r="C19" t="n">
-        <v>3700</v>
+        <v>66600</v>
       </c>
       <c r="D19" t="n">
         <v>0</v>
       </c>
       <c r="E19" t="n">
-        <v>3700</v>
+        <v>66600</v>
       </c>
       <c r="F19" t="n">
-        <v>3700</v>
+        <v>-59200</v>
       </c>
       <c r="G19" t="n">
-        <v>37.00000000000001</v>
+        <v>666</v>
       </c>
       <c r="H19" t="n">
         <v>0</v>
       </c>
       <c r="I19" t="n">
-        <v>37.00000000000001</v>
+        <v>666</v>
       </c>
       <c r="J19" t="inlineStr">
         <is>
@@ -4110,7 +4068,7 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>PARCIAL</t>
+          <t>COMPLETO</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
@@ -4138,21 +4096,21 @@
           <t>{}</t>
         </is>
       </c>
-      <c r="S19" s="7" t="n">
+      <c r="S19" s="6" t="n">
         <v>45875</v>
       </c>
-      <c r="T19" s="7" t="n">
+      <c r="T19" s="6" t="n">
         <v>45875</v>
       </c>
       <c r="U19" t="n">
-        <v>1</v>
-      </c>
-      <c r="V19" s="7" t="n">
-        <v>45987.69726859954</v>
+        <v>18</v>
+      </c>
+      <c r="V19" s="6" t="n">
+        <v>45987.74510344907</v>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>{"Alessandro Cappi": 37.00000000000001}</t>
+          <t>{"Alessandro Cappi": 666.0000000000001}</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
@@ -4171,25 +4129,25 @@
         <v>8300</v>
       </c>
       <c r="C20" t="n">
-        <v>4150</v>
+        <v>74700</v>
       </c>
       <c r="D20" t="n">
         <v>0</v>
       </c>
       <c r="E20" t="n">
-        <v>4150</v>
+        <v>74700</v>
       </c>
       <c r="F20" t="n">
-        <v>4150</v>
+        <v>-66400</v>
       </c>
       <c r="G20" t="n">
-        <v>41.50000000000001</v>
+        <v>747</v>
       </c>
       <c r="H20" t="n">
         <v>0</v>
       </c>
       <c r="I20" t="n">
-        <v>41.50000000000001</v>
+        <v>747</v>
       </c>
       <c r="J20" t="inlineStr">
         <is>
@@ -4198,7 +4156,7 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>PARCIAL</t>
+          <t>COMPLETO</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
@@ -4226,21 +4184,21 @@
           <t>{}</t>
         </is>
       </c>
-      <c r="S20" s="7" t="n">
+      <c r="S20" s="6" t="n">
         <v>45878</v>
       </c>
-      <c r="T20" s="7" t="n">
+      <c r="T20" s="6" t="n">
         <v>45878</v>
       </c>
       <c r="U20" t="n">
-        <v>1</v>
-      </c>
-      <c r="V20" s="7" t="n">
-        <v>45987.69726950231</v>
+        <v>18</v>
+      </c>
+      <c r="V20" s="6" t="n">
+        <v>45987.74510384259</v>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>{"Alessandro Cappi": 41.50000000000001}</t>
+          <t>{"Alessandro Cappi": 747.0000000000001}</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
@@ -4259,25 +4217,25 @@
         <v>9200</v>
       </c>
       <c r="C21" t="n">
-        <v>4600</v>
+        <v>82800</v>
       </c>
       <c r="D21" t="n">
         <v>0</v>
       </c>
       <c r="E21" t="n">
-        <v>4600</v>
+        <v>82800</v>
       </c>
       <c r="F21" t="n">
-        <v>4600</v>
+        <v>-73600</v>
       </c>
       <c r="G21" t="n">
-        <v>46.00000000000001</v>
+        <v>828</v>
       </c>
       <c r="H21" t="n">
         <v>0</v>
       </c>
       <c r="I21" t="n">
-        <v>46.00000000000001</v>
+        <v>828</v>
       </c>
       <c r="J21" t="inlineStr">
         <is>
@@ -4286,7 +4244,7 @@
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>PARCIAL</t>
+          <t>COMPLETO</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
@@ -4314,21 +4272,21 @@
           <t>{}</t>
         </is>
       </c>
-      <c r="S21" s="7" t="n">
+      <c r="S21" s="6" t="n">
         <v>45881</v>
       </c>
-      <c r="T21" s="7" t="n">
+      <c r="T21" s="6" t="n">
         <v>45881</v>
       </c>
       <c r="U21" t="n">
-        <v>1</v>
-      </c>
-      <c r="V21" s="7" t="n">
-        <v>45987.69727054398</v>
+        <v>18</v>
+      </c>
+      <c r="V21" s="6" t="n">
+        <v>45987.74510429398</v>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>{"Alessandro Cappi": 46.00000000000001}</t>
+          <t>{"Alessandro Cappi": 828.0000000000001}</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
@@ -4347,25 +4305,25 @@
         <v>10100</v>
       </c>
       <c r="C22" t="n">
-        <v>5050</v>
+        <v>90900</v>
       </c>
       <c r="D22" t="n">
         <v>0</v>
       </c>
       <c r="E22" t="n">
-        <v>5050</v>
+        <v>90900</v>
       </c>
       <c r="F22" t="n">
-        <v>5050</v>
+        <v>-80800</v>
       </c>
       <c r="G22" t="n">
-        <v>50.50000000000001</v>
+        <v>909</v>
       </c>
       <c r="H22" t="n">
         <v>0</v>
       </c>
       <c r="I22" t="n">
-        <v>50.50000000000001</v>
+        <v>909</v>
       </c>
       <c r="J22" t="inlineStr">
         <is>
@@ -4374,7 +4332,7 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>PARCIAL</t>
+          <t>COMPLETO</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
@@ -4402,21 +4360,21 @@
           <t>{}</t>
         </is>
       </c>
-      <c r="S22" s="7" t="n">
+      <c r="S22" s="6" t="n">
         <v>45884</v>
       </c>
-      <c r="T22" s="7" t="n">
+      <c r="T22" s="6" t="n">
         <v>45884</v>
       </c>
       <c r="U22" t="n">
-        <v>1</v>
-      </c>
-      <c r="V22" s="7" t="n">
-        <v>45987.69727140047</v>
+        <v>18</v>
+      </c>
+      <c r="V22" s="6" t="n">
+        <v>45987.74510469908</v>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>{"Alessandro Cappi": 50.50000000000001}</t>
+          <t>{"Alessandro Cappi": 909.0000000000001}</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
@@ -4435,25 +4393,25 @@
         <v>11000</v>
       </c>
       <c r="C23" t="n">
-        <v>5500</v>
+        <v>99000</v>
       </c>
       <c r="D23" t="n">
         <v>0</v>
       </c>
       <c r="E23" t="n">
-        <v>5500</v>
+        <v>99000</v>
       </c>
       <c r="F23" t="n">
-        <v>5500</v>
+        <v>-88000</v>
       </c>
       <c r="G23" t="n">
-        <v>55.00000000000001</v>
+        <v>990</v>
       </c>
       <c r="H23" t="n">
         <v>0</v>
       </c>
       <c r="I23" t="n">
-        <v>55.00000000000001</v>
+        <v>990</v>
       </c>
       <c r="J23" t="inlineStr">
         <is>
@@ -4462,7 +4420,7 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>PARCIAL</t>
+          <t>COMPLETO</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
@@ -4490,21 +4448,21 @@
           <t>{}</t>
         </is>
       </c>
-      <c r="S23" s="7" t="n">
+      <c r="S23" s="6" t="n">
         <v>45887</v>
       </c>
-      <c r="T23" s="7" t="n">
+      <c r="T23" s="6" t="n">
         <v>45887</v>
       </c>
       <c r="U23" t="n">
-        <v>1</v>
-      </c>
-      <c r="V23" s="7" t="n">
-        <v>45987.69727236111</v>
+        <v>18</v>
+      </c>
+      <c r="V23" s="6" t="n">
+        <v>45987.74510513889</v>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>{"Alessandro Cappi": 55.000000000000014}</t>
+          <t>{"Alessandro Cappi": 990.0000000000001}</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
@@ -4523,25 +4481,25 @@
         <v>11900</v>
       </c>
       <c r="C24" t="n">
-        <v>5950</v>
+        <v>107100</v>
       </c>
       <c r="D24" t="n">
         <v>0</v>
       </c>
       <c r="E24" t="n">
-        <v>5950</v>
+        <v>107100</v>
       </c>
       <c r="F24" t="n">
-        <v>5950</v>
+        <v>-95200</v>
       </c>
       <c r="G24" t="n">
-        <v>59.50000000000001</v>
+        <v>1071</v>
       </c>
       <c r="H24" t="n">
         <v>0</v>
       </c>
       <c r="I24" t="n">
-        <v>59.50000000000001</v>
+        <v>1071</v>
       </c>
       <c r="J24" t="inlineStr">
         <is>
@@ -4550,7 +4508,7 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>PARCIAL</t>
+          <t>COMPLETO</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
@@ -4578,21 +4536,21 @@
           <t>{}</t>
         </is>
       </c>
-      <c r="S24" s="7" t="n">
+      <c r="S24" s="6" t="n">
         <v>45890</v>
       </c>
-      <c r="T24" s="7" t="n">
+      <c r="T24" s="6" t="n">
         <v>45890</v>
       </c>
       <c r="U24" t="n">
-        <v>1</v>
-      </c>
-      <c r="V24" s="7" t="n">
-        <v>45987.69727329861</v>
+        <v>18</v>
+      </c>
+      <c r="V24" s="6" t="n">
+        <v>45987.74510555556</v>
       </c>
       <c r="W24" t="inlineStr">
         <is>
-          <t>{"Alessandro Cappi": 59.500000000000014}</t>
+          <t>{"Alessandro Cappi": 1071.0000000000002}</t>
         </is>
       </c>
       <c r="X24" t="inlineStr">
@@ -4611,25 +4569,25 @@
         <v>12800</v>
       </c>
       <c r="C25" t="n">
-        <v>6400</v>
+        <v>115200</v>
       </c>
       <c r="D25" t="n">
         <v>0</v>
       </c>
       <c r="E25" t="n">
-        <v>6400</v>
+        <v>115200</v>
       </c>
       <c r="F25" t="n">
-        <v>6400</v>
+        <v>-102400</v>
       </c>
       <c r="G25" t="n">
-        <v>64.00000000000001</v>
+        <v>1152</v>
       </c>
       <c r="H25" t="n">
         <v>0</v>
       </c>
       <c r="I25" t="n">
-        <v>64.00000000000001</v>
+        <v>1152</v>
       </c>
       <c r="J25" t="inlineStr">
         <is>
@@ -4638,7 +4596,7 @@
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>PARCIAL</t>
+          <t>COMPLETO</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
@@ -4666,21 +4624,21 @@
           <t>{}</t>
         </is>
       </c>
-      <c r="S25" s="7" t="n">
+      <c r="S25" s="6" t="n">
         <v>45893</v>
       </c>
-      <c r="T25" s="7" t="n">
+      <c r="T25" s="6" t="n">
         <v>45893</v>
       </c>
       <c r="U25" t="n">
-        <v>1</v>
-      </c>
-      <c r="V25" s="7" t="n">
-        <v>45987.69727424769</v>
+        <v>18</v>
+      </c>
+      <c r="V25" s="6" t="n">
+        <v>45987.74510612268</v>
       </c>
       <c r="W25" t="inlineStr">
         <is>
-          <t>{"Alessandro Cappi": 64.00000000000001}</t>
+          <t>{"Alessandro Cappi": 1152.0000000000002}</t>
         </is>
       </c>
       <c r="X25" t="inlineStr">
@@ -4699,25 +4657,25 @@
         <v>13700</v>
       </c>
       <c r="C26" t="n">
-        <v>6850</v>
+        <v>123300</v>
       </c>
       <c r="D26" t="n">
         <v>0</v>
       </c>
       <c r="E26" t="n">
-        <v>6850</v>
+        <v>123300</v>
       </c>
       <c r="F26" t="n">
-        <v>6850</v>
+        <v>-109600</v>
       </c>
       <c r="G26" t="n">
-        <v>68.50000000000001</v>
+        <v>1233</v>
       </c>
       <c r="H26" t="n">
         <v>0</v>
       </c>
       <c r="I26" t="n">
-        <v>68.50000000000001</v>
+        <v>1233</v>
       </c>
       <c r="J26" t="inlineStr">
         <is>
@@ -4726,7 +4684,7 @@
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>PARCIAL</t>
+          <t>COMPLETO</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
@@ -4754,21 +4712,21 @@
           <t>{}</t>
         </is>
       </c>
-      <c r="S26" s="7" t="n">
+      <c r="S26" s="6" t="n">
         <v>45876</v>
       </c>
-      <c r="T26" s="7" t="n">
+      <c r="T26" s="6" t="n">
         <v>45876</v>
       </c>
       <c r="U26" t="n">
-        <v>1</v>
-      </c>
-      <c r="V26" s="7" t="n">
-        <v>45987.69727513889</v>
+        <v>18</v>
+      </c>
+      <c r="V26" s="6" t="n">
+        <v>45987.74510655092</v>
       </c>
       <c r="W26" t="inlineStr">
         <is>
-          <t>{"Alessandro Cappi": 68.50000000000001}</t>
+          <t>{"Alessandro Cappi": 1233.0000000000002}</t>
         </is>
       </c>
       <c r="X26" t="inlineStr">
@@ -4787,25 +4745,25 @@
         <v>14600</v>
       </c>
       <c r="C27" t="n">
-        <v>7300</v>
+        <v>131400</v>
       </c>
       <c r="D27" t="n">
         <v>0</v>
       </c>
       <c r="E27" t="n">
-        <v>7300</v>
+        <v>131400</v>
       </c>
       <c r="F27" t="n">
-        <v>7300</v>
+        <v>-116800</v>
       </c>
       <c r="G27" t="n">
-        <v>73.00000000000001</v>
+        <v>1314</v>
       </c>
       <c r="H27" t="n">
         <v>0</v>
       </c>
       <c r="I27" t="n">
-        <v>73.00000000000001</v>
+        <v>1314</v>
       </c>
       <c r="J27" t="inlineStr">
         <is>
@@ -4814,7 +4772,7 @@
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>PARCIAL</t>
+          <t>COMPLETO</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
@@ -4842,21 +4800,21 @@
           <t>{}</t>
         </is>
       </c>
-      <c r="S27" s="7" t="n">
+      <c r="S27" s="6" t="n">
         <v>45879</v>
       </c>
-      <c r="T27" s="7" t="n">
+      <c r="T27" s="6" t="n">
         <v>45879</v>
       </c>
       <c r="U27" t="n">
-        <v>1</v>
-      </c>
-      <c r="V27" s="7" t="n">
-        <v>45987.69727604167</v>
+        <v>18</v>
+      </c>
+      <c r="V27" s="6" t="n">
+        <v>45987.7451069676</v>
       </c>
       <c r="W27" t="inlineStr">
         <is>
-          <t>{"Alessandro Cappi": 73.00000000000001}</t>
+          <t>{"Alessandro Cappi": 1314.0000000000002}</t>
         </is>
       </c>
       <c r="X27" t="inlineStr">
@@ -4875,25 +4833,25 @@
         <v>15500</v>
       </c>
       <c r="C28" t="n">
-        <v>7750</v>
+        <v>139500</v>
       </c>
       <c r="D28" t="n">
         <v>0</v>
       </c>
       <c r="E28" t="n">
-        <v>7750</v>
+        <v>139500</v>
       </c>
       <c r="F28" t="n">
-        <v>7750</v>
+        <v>-124000</v>
       </c>
       <c r="G28" t="n">
-        <v>77.50000000000001</v>
+        <v>1395</v>
       </c>
       <c r="H28" t="n">
         <v>0</v>
       </c>
       <c r="I28" t="n">
-        <v>77.50000000000001</v>
+        <v>1395</v>
       </c>
       <c r="J28" t="inlineStr">
         <is>
@@ -4902,7 +4860,7 @@
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>PARCIAL</t>
+          <t>COMPLETO</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
@@ -4930,21 +4888,21 @@
           <t>{}</t>
         </is>
       </c>
-      <c r="S28" s="7" t="n">
+      <c r="S28" s="6" t="n">
         <v>45882</v>
       </c>
-      <c r="T28" s="7" t="n">
+      <c r="T28" s="6" t="n">
         <v>45882</v>
       </c>
       <c r="U28" t="n">
-        <v>1</v>
-      </c>
-      <c r="V28" s="7" t="n">
-        <v>45987.69727686342</v>
+        <v>18</v>
+      </c>
+      <c r="V28" s="6" t="n">
+        <v>45987.74510741898</v>
       </c>
       <c r="W28" t="inlineStr">
         <is>
-          <t>{"Alessandro Cappi": 77.50000000000001}</t>
+          <t>{"Alessandro Cappi": 1395.0000000000002}</t>
         </is>
       </c>
       <c r="X28" t="inlineStr">

</xml_diff>